<commit_message>
vault backup: 2026-05-30 23:20:20
</commit_message>
<xml_diff>
--- a/income_forecaster.xlsx
+++ b/income_forecaster.xlsx
@@ -19,6 +19,7 @@
     <sheet name="3-Year Growth" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Pipeline &amp; Capacity" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Leverage Scenarios" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Skyright Sale Scenarios" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="598">
   <si>
     <t xml:space="preserve">Income Forecaster — Chance Peare</t>
   </si>
@@ -1593,6 +1594,237 @@
   </si>
   <si>
     <t xml:space="preserve">• None of these models add a sales hire. If you want &gt; $400K, the next hire is probably a part-time SDR, not another Ops person.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright Sale Scenarios — 24-Month View</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 scenarios: A) Stay at NewCo W2  B) Skyright becomes Embedded retainer  C) Clean exit. Equity payment $125K (editable) at sale month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SALE EVENT INPUTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sale close month (1=Jun26, 5=Oct26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pessimistic: Oct-26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity payment (gross)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5% stake. Mid-low of $100-200K range.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTCG tax rate (federal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15% MFJ for AGI &lt; $583K. Assumes &gt;1-yr holding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity payment (net of tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net cash to bank.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright Embedded retainer rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per CLAUDE.md $6K Embedded tier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright retainer duration (months)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pessimistic: 18 months. New owner installs own ops.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA hire month (timed with sale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct-26. Costs $2K/mo + $400 mgmt overhead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA monthly cost (loaded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct cost + management time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright admin automation savings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours saved on Skyright work via VA + Make automation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours/mo on Skyright Embedded (without leverage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embedded tier standard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours/mo on Skyright Embedded (with VA + automation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective ~21 hrs/mo with VA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO A — Stay at NewCo as W2 COO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright/NewCo W2 ($8K/mo, continues)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity payment (net of LTCG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FW Ops retainer/variable revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO B — Skyright transitions to Embedded retainer (RECOMMENDED PLANNING CASE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright W2 ($8K/mo, ends sale month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright Embedded retainer ($6K/mo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other FW Ops revenue (clients + variable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA cost (loaded, from sale month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total gross income (B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO C — Clean exit (W2 ends, no Skyright relationship)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright W2 (ends sale month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FW Ops revenue (aggressive growth path)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total gross income (C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO COMPARISON SUMMARY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y1 Gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y2 Gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24-Mo Gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active retainers end Y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A — Stay at NewCo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-4 (W2 caps capacity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safe. Equity is bonus. FW Ops grows slowly under W2 demands.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B — Skyright as Embedded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4-5 (incl. Skyright)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best risk-adjusted. $6K/mo + $106K equity + VA leverage. 18-mo Skyright relationship runway.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C — Clean exit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-6 (aggressive)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$106K equity = 12-15 mo runway. Higher acquisition pace possible. Higher risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAPACITY CHECK (Scenario B with VA + automation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skyright Embedded hrs/mo (with VA + automation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reduced from 35 to ~21 hrs/mo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other retainer hrs/mo (3 retainers × 18 hrs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active tier ~18 hrs/mo each.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales hrs/mo (3 closes/yr target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From Pipeline &amp; Capacity tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin + marketing hrs/mo (with VA help)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VA absorbs ~50% of original 52 hrs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL hours/mo required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Available hrs/mo (FT post-sale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same FT capacity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive = fits. Negative = need to drop a retainer or hire more.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRATEGIC NOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Equity tax treatment: assumes LTCG (&gt;1-yr holding). Federal 15% MFJ at AGI &lt;$583K. Verify cost basis with CPA — could be lower than gross if exercised options.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Scenario B (Skyright as Embedded) requires the BUYER to want this arrangement. Most likely if buyer is owner-operator or strategic acquirer who values continuity. PE buyers typically install own ops team — Scenario B unlikely with PE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Skyright Embedded duration (18 months default) is aggressive. Reality: transition retainers often end in 6-12 months once new ops team is in place. Edit Assumptions B10 to test 12-mo case.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• VA hired at sale month to absorb Skyright admin/operational work. Make automations + ServiceTitan integrations + report automation = the 40% time savings on Skyright retainer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• In Scenario B, Skyright becomes both an income source AND your capacity sink. If they need 21 hrs/mo, you only have ~159 hrs/mo for everything else. Tight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Scenario C buys runway with equity but requires faster client acquisition to compensate for lost Skyright income. Aggressive growth path assumes 6 active retainers by end Y2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Equity payment goes into Mercury business account if treated as business income, OR personal if treated as capital gains on personal investment. Most likely the latter (personal LTCG). Confirm with CPA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Health insurance: Scenario A keeps Skyright/NewCo employer coverage. B and C trigger ACA ($1,500-2,500/mo family of 6) starting sale month. NOT modeled here — add $18-30K/yr cost to B and C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tax estimate on Y1 numbers gets complicated: W2 portion withheld, 1099 portion + equity (LTCG) require separate quarterly payments. Cleanup at year-end could be a $10K+ surprise either direction.</t>
   </si>
 </sst>
 </file>
@@ -1792,7 +2024,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="72">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1969,6 +2201,22 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1981,11 +2229,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1993,7 +2237,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2001,11 +2265,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2013,19 +2305,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2882,44 +3166,44 @@
   <dimension ref="A1:F50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="65"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
         <v>396</v>
       </c>
@@ -2939,175 +3223,175 @@
         <v>401</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="C6" s="47" t="n">
+      <c r="C6" s="33" t="n">
         <v>200</v>
       </c>
-      <c r="D6" s="48" t="n">
+      <c r="D6" s="44" t="n">
         <v>60</v>
       </c>
-      <c r="E6" s="48" t="n">
+      <c r="E6" s="44" t="n">
         <v>0.1</v>
       </c>
-      <c r="F6" s="49" t="s">
+      <c r="F6" s="6" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B7" s="50" t="n">
+      <c r="B7" s="36" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="45" t="n">
         <f aca="false">C6*B7</f>
         <v>20</v>
       </c>
-      <c r="D7" s="52" t="n">
+      <c r="D7" s="42" t="n">
         <f aca="false">D6*0.25</f>
         <v>15</v>
       </c>
-      <c r="F7" s="49" t="s">
+      <c r="F7" s="6" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B8" s="50" t="n">
+      <c r="B8" s="36" t="n">
         <v>0.35</v>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="45" t="n">
         <f aca="false">C7*B8</f>
         <v>7</v>
       </c>
-      <c r="D8" s="52" t="n">
+      <c r="D8" s="42" t="n">
         <f aca="false">D7*0.45</f>
         <v>6.75</v>
       </c>
-      <c r="E8" s="48" t="n">
+      <c r="E8" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="49" t="s">
+      <c r="F8" s="6" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B9" s="50" t="n">
+      <c r="B9" s="36" t="n">
         <v>0.55</v>
       </c>
-      <c r="C9" s="51" t="n">
+      <c r="C9" s="45" t="n">
         <f aca="false">C8*B9</f>
         <v>3.85</v>
       </c>
-      <c r="D9" s="52" t="n">
+      <c r="D9" s="42" t="n">
         <f aca="false">D8*0.6</f>
         <v>4.05</v>
       </c>
-      <c r="E9" s="48" t="n">
+      <c r="E9" s="44" t="n">
         <v>6</v>
       </c>
-      <c r="F9" s="49" t="s">
+      <c r="F9" s="6" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B10" s="50" t="n">
+      <c r="B10" s="36" t="n">
         <v>0.75</v>
       </c>
-      <c r="C10" s="51" t="n">
+      <c r="C10" s="45" t="n">
         <f aca="false">C9*B10</f>
         <v>2.8875</v>
       </c>
-      <c r="D10" s="52" t="n">
+      <c r="D10" s="42" t="n">
         <f aca="false">D9*0.8</f>
         <v>3.24</v>
       </c>
-      <c r="E10" s="48" t="n">
+      <c r="E10" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="49" t="s">
+      <c r="F10" s="6" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B11" s="50" t="n">
+      <c r="B11" s="36" t="n">
         <v>0.35</v>
       </c>
-      <c r="C11" s="51" t="n">
+      <c r="C11" s="45" t="n">
         <f aca="false">C10*B11</f>
         <v>1.010625</v>
       </c>
-      <c r="D11" s="52" t="n">
+      <c r="D11" s="42" t="n">
         <f aca="false">D10*0.4</f>
         <v>1.296</v>
       </c>
-      <c r="E11" s="48" t="n">
+      <c r="E11" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="6" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="46"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B14" s="53" t="n">
+      <c r="B14" s="46" t="n">
         <f aca="false">6+(C7*E7)+(C8*E8)+(C9*E9)+(C10*E10)+(C11*E11)</f>
         <v>57.681875</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="B15" s="53" t="n">
+      <c r="B15" s="46" t="n">
         <f aca="false">3+(D7*E7)+(D8*E8)+(D9*E9)+(D10*E10)+(D11*E11)</f>
         <v>57.648</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
         <v>420</v>
       </c>
@@ -3124,210 +3408,210 @@
         <v>424</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="54" t="n">
+      <c r="B19" s="41" t="n">
         <f aca="false">2*B14</f>
         <v>115.36375</v>
       </c>
-      <c r="C19" s="54" t="n">
+      <c r="C19" s="41" t="n">
         <f aca="false">2*B15</f>
         <v>115.296</v>
       </c>
-      <c r="D19" s="54" t="n">
+      <c r="D19" s="41" t="n">
         <f aca="false">AVERAGE(B19:C19)</f>
         <v>115.329875</v>
       </c>
-      <c r="E19" s="52" t="n">
+      <c r="E19" s="42" t="n">
         <f aca="false">D19/48</f>
         <v>2.40270572916667</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="54" t="n">
+      <c r="B20" s="41" t="n">
         <f aca="false">3*B14</f>
         <v>173.045625</v>
       </c>
-      <c r="C20" s="54" t="n">
+      <c r="C20" s="41" t="n">
         <f aca="false">3*B15</f>
         <v>172.944</v>
       </c>
-      <c r="D20" s="54" t="n">
+      <c r="D20" s="41" t="n">
         <f aca="false">AVERAGE(B20:C20)</f>
         <v>172.9948125</v>
       </c>
-      <c r="E20" s="52" t="n">
+      <c r="E20" s="42" t="n">
         <f aca="false">D20/48</f>
         <v>3.60405859375</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B21" s="54" t="n">
+      <c r="B21" s="41" t="n">
         <f aca="false">4*B14</f>
         <v>230.7275</v>
       </c>
-      <c r="C21" s="54" t="n">
+      <c r="C21" s="41" t="n">
         <f aca="false">4*B15</f>
         <v>230.592</v>
       </c>
-      <c r="D21" s="54" t="n">
+      <c r="D21" s="41" t="n">
         <f aca="false">AVERAGE(B21:C21)</f>
         <v>230.65975</v>
       </c>
-      <c r="E21" s="52" t="n">
+      <c r="E21" s="42" t="n">
         <f aca="false">D21/48</f>
         <v>4.80541145833333</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B22" s="54" t="n">
+      <c r="B22" s="41" t="n">
         <f aca="false">5*B14</f>
         <v>288.409375</v>
       </c>
-      <c r="C22" s="54" t="n">
+      <c r="C22" s="41" t="n">
         <f aca="false">5*B15</f>
         <v>288.24</v>
       </c>
-      <c r="D22" s="54" t="n">
+      <c r="D22" s="41" t="n">
         <f aca="false">AVERAGE(B22:C22)</f>
         <v>288.3246875</v>
       </c>
-      <c r="E22" s="52" t="n">
+      <c r="E22" s="42" t="n">
         <f aca="false">D22/48</f>
         <v>6.00676432291667</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B23" s="54" t="n">
+      <c r="B23" s="41" t="n">
         <f aca="false">6*B14</f>
         <v>346.09125</v>
       </c>
-      <c r="C23" s="54" t="n">
+      <c r="C23" s="41" t="n">
         <f aca="false">6*B15</f>
         <v>345.888</v>
       </c>
-      <c r="D23" s="54" t="n">
+      <c r="D23" s="41" t="n">
         <f aca="false">AVERAGE(B23:C23)</f>
         <v>345.989625</v>
       </c>
-      <c r="E23" s="52" t="n">
+      <c r="E23" s="42" t="n">
         <f aca="false">D23/48</f>
         <v>7.2081171875</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="46" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>425</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="B26" s="47" t="n">
+      <c r="B26" s="33" t="n">
         <v>45</v>
       </c>
-      <c r="F26" s="49" t="s">
+      <c r="F26" s="6" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B27" s="47" t="n">
+      <c r="B27" s="33" t="n">
         <v>48</v>
       </c>
-      <c r="F27" s="49" t="s">
+      <c r="F27" s="6" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B28" s="51" t="n">
+      <c r="B28" s="45" t="n">
         <f aca="false">B26*B27</f>
         <v>2160</v>
       </c>
-      <c r="F28" s="49" t="s">
+      <c r="F28" s="6" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="B29" s="47" t="n">
+      <c r="B29" s="33" t="n">
         <v>18</v>
       </c>
-      <c r="F29" s="49" t="s">
+      <c r="F29" s="6" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B30" s="47" t="n">
+      <c r="B30" s="33" t="n">
         <v>35</v>
       </c>
-      <c r="F30" s="49" t="s">
+      <c r="F30" s="6" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="B31" s="47" t="n">
+      <c r="B31" s="33" t="n">
         <v>32</v>
       </c>
-      <c r="F31" s="49" t="s">
+      <c r="F31" s="6" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B32" s="47" t="n">
+      <c r="B32" s="33" t="n">
         <v>20</v>
       </c>
-      <c r="F32" s="49" t="s">
+      <c r="F32" s="6" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="46" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>440</v>
       </c>
-      <c r="B34" s="46"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="46"/>
-      <c r="F34" s="46"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="30" t="s">
         <v>441</v>
       </c>
@@ -3347,133 +3631,133 @@
         <v>401</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B36" s="47" t="n">
+      <c r="B36" s="33" t="n">
         <v>50</v>
       </c>
-      <c r="C36" s="54" t="n">
+      <c r="C36" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="D36" s="54" t="n">
+      <c r="D36" s="41" t="n">
         <f aca="false">B36-C36-15-5</f>
         <v>20</v>
       </c>
-      <c r="E36" s="54" t="n">
+      <c r="E36" s="41" t="n">
         <f aca="false">ROUNDDOWN(D36/B29,0)</f>
         <v>1</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="F36" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B37" s="54" t="n">
+      <c r="B37" s="41" t="n">
         <f aca="false">B28/12</f>
         <v>180</v>
       </c>
-      <c r="C37" s="54" t="n">
+      <c r="C37" s="41" t="n">
         <f aca="false">AVERAGE(D19:D22)/12</f>
         <v>16.8189401041667</v>
       </c>
-      <c r="D37" s="54" t="n">
+      <c r="D37" s="41" t="n">
         <f aca="false">B37-C37-B31-B32</f>
         <v>111.181059895833</v>
       </c>
-      <c r="E37" s="54" t="n">
+      <c r="E37" s="41" t="n">
         <f aca="false">ROUNDDOWN(D37/B29,0)</f>
         <v>6</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="F37" s="1" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B38" s="54" t="n">
+      <c r="B38" s="41" t="n">
         <f aca="false">B28/12</f>
         <v>180</v>
       </c>
-      <c r="C38" s="54" t="n">
+      <c r="C38" s="41" t="n">
         <f aca="false">AVERAGE(D19:D22)/12*0.5</f>
         <v>8.40947005208333</v>
       </c>
-      <c r="D38" s="54" t="n">
+      <c r="D38" s="41" t="n">
         <f aca="false">B38-C38-B31*0.3-B32*0.4</f>
         <v>153.990529947917</v>
       </c>
-      <c r="E38" s="54" t="n">
+      <c r="E38" s="41" t="n">
         <f aca="false">ROUNDDOWN(D38/B29,0)</f>
         <v>8</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="F38" s="1" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B39" s="54" t="n">
+      <c r="B39" s="41" t="n">
         <f aca="false">B28/12</f>
         <v>180</v>
       </c>
-      <c r="C39" s="54" t="n">
+      <c r="C39" s="41" t="n">
         <f aca="false">AVERAGE(D19:D22)/12*0.35</f>
         <v>5.88662903645833</v>
       </c>
-      <c r="D39" s="54" t="n">
+      <c r="D39" s="41" t="n">
         <f aca="false">B39-C39-B31*0.2-B32*0.3</f>
         <v>161.713370963542</v>
       </c>
-      <c r="E39" s="54" t="n">
+      <c r="E39" s="41" t="n">
         <f aca="false">ROUNDDOWN(D39/B29,0)</f>
         <v>8</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="F39" s="1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B40" s="54" t="n">
+      <c r="B40" s="41" t="n">
         <f aca="false">B28/12</f>
         <v>180</v>
       </c>
-      <c r="C40" s="54" t="n">
+      <c r="C40" s="41" t="n">
         <f aca="false">AVERAGE(D19:D22)/12*0.25</f>
         <v>4.20473502604167</v>
       </c>
-      <c r="D40" s="54" t="n">
+      <c r="D40" s="41" t="n">
         <f aca="false">B40-C40-B31*0.15-B32*0.25</f>
         <v>165.995264973958</v>
       </c>
-      <c r="E40" s="54" t="n">
+      <c r="E40" s="41" t="n">
         <f aca="false">ROUNDDOWN(D40/B29,0)</f>
         <v>9</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="F40" s="1" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="46" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="27" t="s">
@@ -3592,161 +3876,161 @@
   <dimension ref="A1:I52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>466</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="B5" s="55" t="n">
+      <c r="B5" s="15" t="n">
         <v>2000</v>
       </c>
-      <c r="C5" s="49" t="s">
+      <c r="C5" s="6" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="B6" s="55" t="n">
+      <c r="B6" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="C6" s="6" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="B7" s="55" t="n">
+      <c r="B7" s="15" t="n">
         <v>4000</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="6" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="B8" s="55" t="n">
+      <c r="B8" s="15" t="n">
         <v>600</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="6" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="B9" s="55" t="n">
+      <c r="B9" s="15" t="n">
         <v>6583</v>
       </c>
-      <c r="C9" s="49" t="s">
+      <c r="C9" s="6" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="B10" s="55" t="n">
+      <c r="B10" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="C10" s="49" t="s">
+      <c r="C10" s="6" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="B11" s="55" t="n">
+      <c r="B11" s="15" t="n">
         <v>7833</v>
       </c>
-      <c r="C11" s="49" t="s">
+      <c r="C11" s="6" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="B12" s="55" t="n">
+      <c r="B12" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="C12" s="49"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="B13" s="55" t="n">
+      <c r="B13" s="15" t="n">
         <v>1100</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="6" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="46" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
         <v>486</v>
       </c>
@@ -3766,120 +4050,120 @@
         <v>491</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="B17" s="56" t="n">
+      <c r="B17" s="47" t="n">
         <f aca="false">IF(180000&lt;=180000,180000-12*$B$13,"OVER CAP")</f>
         <v>166800</v>
       </c>
-      <c r="C17" s="56" t="n">
+      <c r="C17" s="47" t="n">
         <f aca="false">IF(180000&lt;=252000,180000-12*($B$5+$B$6)-12*$B$13,"OVER CAP")</f>
         <v>138000</v>
       </c>
-      <c r="D17" s="56" t="n">
+      <c r="D17" s="47" t="n">
         <f aca="false">IF(180000&lt;=288000,180000-12*($B$7+$B$8)-12*$B$13,"OVER CAP")</f>
         <v>111600</v>
       </c>
-      <c r="E17" s="56" t="n">
+      <c r="E17" s="47" t="n">
         <f aca="false">IF(180000&lt;=324000,180000-12*($B$9+$B$10)-12*$B$13,"OVER CAP")</f>
         <v>83004</v>
       </c>
-      <c r="F17" s="56" t="n">
+      <c r="F17" s="47" t="n">
         <f aca="false">IF(180000&lt;=400000,180000-12*($B$11+$B$12)-12*$B$13,"OVER CAP")</f>
         <v>68004</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="B18" s="56" t="str">
+      <c r="B18" s="47" t="str">
         <f aca="false">IF(230000&lt;=180000,230000-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C18" s="56" t="n">
+      <c r="C18" s="47" t="n">
         <f aca="false">IF(230000&lt;=252000,230000-12*($B$5+$B$6)-12*$B$13,"OVER CAP")</f>
         <v>188000</v>
       </c>
-      <c r="D18" s="56" t="n">
+      <c r="D18" s="47" t="n">
         <f aca="false">IF(230000&lt;=288000,230000-12*($B$7+$B$8)-12*$B$13,"OVER CAP")</f>
         <v>161600</v>
       </c>
-      <c r="E18" s="56" t="n">
+      <c r="E18" s="47" t="n">
         <f aca="false">IF(230000&lt;=324000,230000-12*($B$9+$B$10)-12*$B$13,"OVER CAP")</f>
         <v>133004</v>
       </c>
-      <c r="F18" s="56" t="n">
+      <c r="F18" s="47" t="n">
         <f aca="false">IF(230000&lt;=400000,230000-12*($B$11+$B$12)-12*$B$13,"OVER CAP")</f>
         <v>118004</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="B19" s="56" t="str">
+      <c r="B19" s="47" t="str">
         <f aca="false">IF(280000&lt;=180000,280000-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C19" s="56" t="str">
+      <c r="C19" s="47" t="str">
         <f aca="false">IF(280000&lt;=252000,280000-12*($B$5+$B$6)-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="D19" s="56" t="n">
+      <c r="D19" s="47" t="n">
         <f aca="false">IF(280000&lt;=288000,280000-12*($B$7+$B$8)-12*$B$13,"OVER CAP")</f>
         <v>211600</v>
       </c>
-      <c r="E19" s="56" t="n">
+      <c r="E19" s="47" t="n">
         <f aca="false">IF(280000&lt;=324000,280000-12*($B$9+$B$10)-12*$B$13,"OVER CAP")</f>
         <v>183004</v>
       </c>
-      <c r="F19" s="56" t="n">
+      <c r="F19" s="47" t="n">
         <f aca="false">IF(280000&lt;=400000,280000-12*($B$11+$B$12)-12*$B$13,"OVER CAP")</f>
         <v>168004</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="B20" s="56" t="str">
+      <c r="B20" s="47" t="str">
         <f aca="false">IF(350000&lt;=180000,350000-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C20" s="56" t="str">
+      <c r="C20" s="47" t="str">
         <f aca="false">IF(350000&lt;=252000,350000-12*($B$5+$B$6)-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="D20" s="56" t="str">
+      <c r="D20" s="47" t="str">
         <f aca="false">IF(350000&lt;=288000,350000-12*($B$7+$B$8)-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="E20" s="56" t="str">
+      <c r="E20" s="47" t="str">
         <f aca="false">IF(350000&lt;=324000,350000-12*($B$9+$B$10)-12*$B$13,"OVER CAP")</f>
         <v>OVER CAP</v>
       </c>
-      <c r="F20" s="56" t="n">
+      <c r="F20" s="47" t="n">
         <f aca="false">IF(350000&lt;=400000,350000-12*($B$11+$B$12)-12*$B$13,"OVER CAP")</f>
         <v>238004</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>496</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="30" t="s">
         <v>486</v>
       </c>
@@ -3899,120 +4183,120 @@
         <v>500</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="B24" s="57" t="n">
+      <c r="B24" s="18" t="n">
         <f aca="false">B17</f>
         <v>166800</v>
       </c>
-      <c r="C24" s="57" t="n">
+      <c r="C24" s="18" t="n">
         <f aca="false">IFERROR(C17-B17, "")</f>
         <v>-28800</v>
       </c>
-      <c r="D24" s="57" t="n">
+      <c r="D24" s="18" t="n">
         <f aca="false">IFERROR(D17-B17, "")</f>
         <v>-55200</v>
       </c>
-      <c r="E24" s="57" t="n">
+      <c r="E24" s="18" t="n">
         <f aca="false">IFERROR(E17-B17, "")</f>
         <v>-83796</v>
       </c>
-      <c r="F24" s="57" t="n">
+      <c r="F24" s="18" t="n">
         <f aca="false">IFERROR(F17-B17, "")</f>
         <v>-98796</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="B25" s="57" t="str">
+      <c r="B25" s="18" t="str">
         <f aca="false">B18</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C25" s="57" t="str">
+      <c r="C25" s="18" t="str">
         <f aca="false">IFERROR(C18-B18, "")</f>
         <v/>
       </c>
-      <c r="D25" s="57" t="str">
+      <c r="D25" s="18" t="str">
         <f aca="false">IFERROR(D18-B18, "")</f>
         <v/>
       </c>
-      <c r="E25" s="57" t="str">
+      <c r="E25" s="18" t="str">
         <f aca="false">IFERROR(E18-B18, "")</f>
         <v/>
       </c>
-      <c r="F25" s="57" t="str">
+      <c r="F25" s="18" t="str">
         <f aca="false">IFERROR(F18-B18, "")</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="B26" s="57" t="str">
+      <c r="B26" s="18" t="str">
         <f aca="false">B19</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C26" s="57" t="str">
+      <c r="C26" s="18" t="str">
         <f aca="false">IFERROR(C19-B19, "")</f>
         <v/>
       </c>
-      <c r="D26" s="57" t="str">
+      <c r="D26" s="18" t="str">
         <f aca="false">IFERROR(D19-B19, "")</f>
         <v/>
       </c>
-      <c r="E26" s="57" t="str">
+      <c r="E26" s="18" t="str">
         <f aca="false">IFERROR(E19-B19, "")</f>
         <v/>
       </c>
-      <c r="F26" s="57" t="str">
+      <c r="F26" s="18" t="str">
         <f aca="false">IFERROR(F19-B19, "")</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="B27" s="57" t="str">
+      <c r="B27" s="18" t="str">
         <f aca="false">B20</f>
         <v>OVER CAP</v>
       </c>
-      <c r="C27" s="57" t="str">
+      <c r="C27" s="18" t="str">
         <f aca="false">IFERROR(C20-B20, "")</f>
         <v/>
       </c>
-      <c r="D27" s="57" t="str">
+      <c r="D27" s="18" t="str">
         <f aca="false">IFERROR(D20-B20, "")</f>
         <v/>
       </c>
-      <c r="E27" s="57" t="str">
+      <c r="E27" s="18" t="str">
         <f aca="false">IFERROR(E20-B20, "")</f>
         <v/>
       </c>
-      <c r="F27" s="57" t="str">
+      <c r="F27" s="18" t="str">
         <f aca="false">IFERROR(F20-B20, "")</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="46" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
         <v>501</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="30" t="s">
         <v>502</v>
       </c>
@@ -4026,86 +4310,86 @@
         <v>505</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="B32" s="58" t="n">
+      <c r="B32" s="38" t="n">
         <f aca="false">12*($B$5+$B$6)</f>
         <v>28800</v>
       </c>
-      <c r="C32" s="58" t="n">
+      <c r="C32" s="38" t="n">
         <f aca="false">B32+600*ROUNDUP(B32/36000,0)</f>
         <v>29400</v>
       </c>
-      <c r="D32" s="52" t="n">
+      <c r="D32" s="42" t="n">
         <f aca="false">ROUNDUP(B32/36000,1)</f>
         <v>0.8</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="B33" s="58" t="n">
+      <c r="B33" s="38" t="n">
         <f aca="false">12*($B$7+$B$8)</f>
         <v>55200</v>
       </c>
-      <c r="C33" s="58" t="n">
+      <c r="C33" s="38" t="n">
         <f aca="false">B33+600*ROUNDUP(B33/36000,0)</f>
         <v>56400</v>
       </c>
-      <c r="D33" s="52" t="n">
+      <c r="D33" s="42" t="n">
         <f aca="false">ROUNDUP(B33/36000,1)</f>
         <v>1.6</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="B34" s="58" t="n">
+      <c r="B34" s="38" t="n">
         <f aca="false">12*($B$9+$B$10)</f>
         <v>83796</v>
       </c>
-      <c r="C34" s="58" t="n">
+      <c r="C34" s="38" t="n">
         <f aca="false">B34+600*ROUNDUP(B34/36000,0)</f>
         <v>85596</v>
       </c>
-      <c r="D34" s="52" t="n">
+      <c r="D34" s="42" t="n">
         <f aca="false">ROUNDUP(B34/36000,1)</f>
         <v>2.4</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="B35" s="58" t="n">
+      <c r="B35" s="38" t="n">
         <f aca="false">12*($B$11+$B$12)</f>
         <v>98796</v>
       </c>
-      <c r="C35" s="58" t="n">
+      <c r="C35" s="38" t="n">
         <f aca="false">B35+600*ROUNDUP(B35/36000,0)</f>
         <v>100596</v>
       </c>
-      <c r="D35" s="52" t="n">
+      <c r="D35" s="42" t="n">
         <f aca="false">ROUNDUP(B35/36000,1)</f>
         <v>2.8</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="46" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="27" t="s">
@@ -4120,7 +4404,7 @@
       <c r="H39" s="27"/>
       <c r="I39" s="27"/>
     </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="27" t="s">
         <v>510</v>
       </c>
@@ -4146,7 +4430,7 @@
       <c r="H41" s="27"/>
       <c r="I41" s="27"/>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="27" t="s">
         <v>512</v>
       </c>
@@ -4159,7 +4443,7 @@
       <c r="H42" s="27"/>
       <c r="I42" s="27"/>
     </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="27" t="s">
         <v>513</v>
       </c>
@@ -4172,20 +4456,20 @@
       <c r="H43" s="27"/>
       <c r="I43" s="27"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="46" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>514</v>
       </c>
-      <c r="B46" s="46"/>
-      <c r="C46" s="46"/>
-      <c r="D46" s="46"/>
-      <c r="E46" s="46"/>
-      <c r="F46" s="46"/>
-      <c r="G46" s="46"/>
-      <c r="H46" s="46"/>
-      <c r="I46" s="46"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="27" t="s">
         <v>515</v>
       </c>
@@ -4224,7 +4508,7 @@
       <c r="H49" s="27"/>
       <c r="I49" s="27"/>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="27" t="s">
         <v>518</v>
       </c>
@@ -4237,7 +4521,7 @@
       <c r="H50" s="27"/>
       <c r="I50" s="27"/>
     </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="27" t="s">
         <v>519</v>
       </c>
@@ -4284,6 +4568,2339 @@
     <mergeCell ref="A50:I50"/>
     <mergeCell ref="A51:I51"/>
     <mergeCell ref="A52:I52"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AB64"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="48" t="s">
+        <v>521</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="48"/>
+      <c r="W1" s="48"/>
+      <c r="X1" s="48"/>
+      <c r="Y1" s="48"/>
+      <c r="Z1" s="48"/>
+      <c r="AA1" s="48"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+      <c r="S2" s="49"/>
+      <c r="T2" s="49"/>
+      <c r="U2" s="49"/>
+      <c r="V2" s="49"/>
+      <c r="W2" s="49"/>
+      <c r="X2" s="49"/>
+      <c r="Y2" s="49"/>
+      <c r="Z2" s="49"/>
+      <c r="AA2" s="49"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="50" t="s">
+        <v>523</v>
+      </c>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>524</v>
+      </c>
+      <c r="B5" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>526</v>
+      </c>
+      <c r="B6" s="53" t="n">
+        <v>125000</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>528</v>
+      </c>
+      <c r="B7" s="54" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>530</v>
+      </c>
+      <c r="B8" s="55" t="n">
+        <f aca="false">B6*(1-B7)</f>
+        <v>106250</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>532</v>
+      </c>
+      <c r="B9" s="56" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>534</v>
+      </c>
+      <c r="B10" s="51" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>536</v>
+      </c>
+      <c r="B11" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>538</v>
+      </c>
+      <c r="B12" s="56" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>540</v>
+      </c>
+      <c r="B13" s="57" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C13" s="52" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>542</v>
+      </c>
+      <c r="B14" s="58" t="n">
+        <v>35</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>544</v>
+      </c>
+      <c r="B15" s="59" t="n">
+        <f aca="false">B14*(1-B13)</f>
+        <v>21</v>
+      </c>
+      <c r="C15" s="52" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="G17" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="H17" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="I17" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="K17" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="L17" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="M17" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="N17" s="30" t="s">
+        <v>321</v>
+      </c>
+      <c r="O17" s="30" t="s">
+        <v>322</v>
+      </c>
+      <c r="P17" s="30" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q17" s="30" t="s">
+        <v>324</v>
+      </c>
+      <c r="R17" s="30" t="s">
+        <v>325</v>
+      </c>
+      <c r="S17" s="30" t="s">
+        <v>326</v>
+      </c>
+      <c r="T17" s="30" t="s">
+        <v>327</v>
+      </c>
+      <c r="U17" s="30" t="s">
+        <v>328</v>
+      </c>
+      <c r="V17" s="30" t="s">
+        <v>329</v>
+      </c>
+      <c r="W17" s="30" t="s">
+        <v>330</v>
+      </c>
+      <c r="X17" s="30" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y17" s="30" t="s">
+        <v>332</v>
+      </c>
+      <c r="Z17" s="60" t="s">
+        <v>345</v>
+      </c>
+      <c r="AA17" s="60" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="50" t="s">
+        <v>546</v>
+      </c>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="Q19" s="50"/>
+      <c r="R19" s="50"/>
+      <c r="S19" s="50"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="50"/>
+      <c r="V19" s="50"/>
+      <c r="W19" s="50"/>
+      <c r="X19" s="50"/>
+      <c r="Y19" s="50"/>
+      <c r="Z19" s="50"/>
+      <c r="AA19" s="50"/>
+      <c r="AB19" s="50"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>547</v>
+      </c>
+      <c r="B20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="K20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="M20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="N20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="O20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="Q20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="R20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="S20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="T20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="U20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="V20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="W20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="X20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="Y20" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="Z20" s="55" t="n">
+        <f aca="false">SUM(B20:M20)</f>
+        <v>96000</v>
+      </c>
+      <c r="AA20" s="55" t="n">
+        <f aca="false">SUM(N20:Y20)</f>
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>548</v>
+      </c>
+      <c r="B21" s="61" t="n">
+        <f aca="false">IF(1=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="61" t="n">
+        <f aca="false">IF(2=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="61" t="n">
+        <f aca="false">IF(3=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="61" t="n">
+        <f aca="false">IF(4=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="61" t="n">
+        <f aca="false">IF(5=$B$5,$B$8,0)</f>
+        <v>106250</v>
+      </c>
+      <c r="G21" s="61" t="n">
+        <f aca="false">IF(6=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="61" t="n">
+        <f aca="false">IF(7=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="61" t="n">
+        <f aca="false">IF(8=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="61" t="n">
+        <f aca="false">IF(9=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="61" t="n">
+        <f aca="false">IF(10=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="61" t="n">
+        <f aca="false">IF(11=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="61" t="n">
+        <f aca="false">IF(12=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="61" t="n">
+        <f aca="false">IF(13=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O21" s="61" t="n">
+        <f aca="false">IF(14=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P21" s="61" t="n">
+        <f aca="false">IF(15=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="61" t="n">
+        <f aca="false">IF(16=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R21" s="61" t="n">
+        <f aca="false">IF(17=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S21" s="61" t="n">
+        <f aca="false">IF(18=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T21" s="61" t="n">
+        <f aca="false">IF(19=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U21" s="61" t="n">
+        <f aca="false">IF(20=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V21" s="61" t="n">
+        <f aca="false">IF(21=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W21" s="61" t="n">
+        <f aca="false">IF(22=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X21" s="61" t="n">
+        <f aca="false">IF(23=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y21" s="61" t="n">
+        <f aca="false">IF(24=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z21" s="55" t="n">
+        <f aca="false">SUM(B21:M21)</f>
+        <v>106250</v>
+      </c>
+      <c r="AA21" s="55" t="n">
+        <f aca="false">SUM(N21:Y21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>549</v>
+      </c>
+      <c r="B22" s="61" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C22" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D22" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E22" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F22" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G22" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H22" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="J22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="K22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="L22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="M22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="N22" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="O22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="P22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="Q22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="R22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="S22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="T22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="U22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="V22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="W22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="X22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="Y22" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="Z22" s="55" t="n">
+        <f aca="false">SUM(B22:M22)</f>
+        <v>98000</v>
+      </c>
+      <c r="AA22" s="55" t="n">
+        <f aca="false">SUM(N22:Y22)</f>
+        <v>159000</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="62" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23" s="63" t="n">
+        <f aca="false">B20+B21+B22</f>
+        <v>11500</v>
+      </c>
+      <c r="C23" s="63" t="n">
+        <f aca="false">C20+C21+C22</f>
+        <v>13000</v>
+      </c>
+      <c r="D23" s="63" t="n">
+        <f aca="false">D20+D21+D22</f>
+        <v>13000</v>
+      </c>
+      <c r="E23" s="63" t="n">
+        <f aca="false">E20+E21+E22</f>
+        <v>16000</v>
+      </c>
+      <c r="F23" s="63" t="n">
+        <f aca="false">F20+F21+F22</f>
+        <v>122250</v>
+      </c>
+      <c r="G23" s="63" t="n">
+        <f aca="false">G20+G21+G22</f>
+        <v>16000</v>
+      </c>
+      <c r="H23" s="63" t="n">
+        <f aca="false">H20+H21+H22</f>
+        <v>16000</v>
+      </c>
+      <c r="I23" s="63" t="n">
+        <f aca="false">I20+I21+I22</f>
+        <v>18500</v>
+      </c>
+      <c r="J23" s="63" t="n">
+        <f aca="false">J20+J21+J22</f>
+        <v>18500</v>
+      </c>
+      <c r="K23" s="63" t="n">
+        <f aca="false">K20+K21+K22</f>
+        <v>18500</v>
+      </c>
+      <c r="L23" s="63" t="n">
+        <f aca="false">L20+L21+L22</f>
+        <v>18500</v>
+      </c>
+      <c r="M23" s="63" t="n">
+        <f aca="false">M20+M21+M22</f>
+        <v>18500</v>
+      </c>
+      <c r="N23" s="63" t="n">
+        <f aca="false">N20+N21+N22</f>
+        <v>18500</v>
+      </c>
+      <c r="O23" s="63" t="n">
+        <f aca="false">O20+O21+O22</f>
+        <v>21500</v>
+      </c>
+      <c r="P23" s="63" t="n">
+        <f aca="false">P20+P21+P22</f>
+        <v>21500</v>
+      </c>
+      <c r="Q23" s="63" t="n">
+        <f aca="false">Q20+Q21+Q22</f>
+        <v>21500</v>
+      </c>
+      <c r="R23" s="63" t="n">
+        <f aca="false">R20+R21+R22</f>
+        <v>21500</v>
+      </c>
+      <c r="S23" s="63" t="n">
+        <f aca="false">S20+S21+S22</f>
+        <v>21500</v>
+      </c>
+      <c r="T23" s="63" t="n">
+        <f aca="false">T20+T21+T22</f>
+        <v>21500</v>
+      </c>
+      <c r="U23" s="63" t="n">
+        <f aca="false">U20+U21+U22</f>
+        <v>21500</v>
+      </c>
+      <c r="V23" s="63" t="n">
+        <f aca="false">V20+V21+V22</f>
+        <v>21500</v>
+      </c>
+      <c r="W23" s="63" t="n">
+        <f aca="false">W20+W21+W22</f>
+        <v>21500</v>
+      </c>
+      <c r="X23" s="63" t="n">
+        <f aca="false">X20+X21+X22</f>
+        <v>21500</v>
+      </c>
+      <c r="Y23" s="63" t="n">
+        <f aca="false">Y20+Y21+Y22</f>
+        <v>21500</v>
+      </c>
+      <c r="Z23" s="63" t="n">
+        <f aca="false">SUM(B23:M23)</f>
+        <v>300250</v>
+      </c>
+      <c r="AA23" s="63" t="n">
+        <f aca="false">SUM(N23:Y23)</f>
+        <v>255000</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="50" t="s">
+        <v>550</v>
+      </c>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
+      <c r="O25" s="50"/>
+      <c r="P25" s="50"/>
+      <c r="Q25" s="50"/>
+      <c r="R25" s="50"/>
+      <c r="S25" s="50"/>
+      <c r="T25" s="50"/>
+      <c r="U25" s="50"/>
+      <c r="V25" s="50"/>
+      <c r="W25" s="50"/>
+      <c r="X25" s="50"/>
+      <c r="Y25" s="50"/>
+      <c r="Z25" s="50"/>
+      <c r="AA25" s="50"/>
+      <c r="AB25" s="50"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>551</v>
+      </c>
+      <c r="B26" s="61" t="n">
+        <f aca="false">IF(1&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="C26" s="61" t="n">
+        <f aca="false">IF(2&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="D26" s="61" t="n">
+        <f aca="false">IF(3&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="E26" s="61" t="n">
+        <f aca="false">IF(4&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="F26" s="61" t="n">
+        <f aca="false">IF(5&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="61" t="n">
+        <f aca="false">IF(6&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="61" t="n">
+        <f aca="false">IF(7&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="61" t="n">
+        <f aca="false">IF(8&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="61" t="n">
+        <f aca="false">IF(9&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="61" t="n">
+        <f aca="false">IF(10&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L26" s="61" t="n">
+        <f aca="false">IF(11&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M26" s="61" t="n">
+        <f aca="false">IF(12&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N26" s="61" t="n">
+        <f aca="false">IF(13&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O26" s="61" t="n">
+        <f aca="false">IF(14&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P26" s="61" t="n">
+        <f aca="false">IF(15&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q26" s="61" t="n">
+        <f aca="false">IF(16&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R26" s="61" t="n">
+        <f aca="false">IF(17&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S26" s="61" t="n">
+        <f aca="false">IF(18&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T26" s="61" t="n">
+        <f aca="false">IF(19&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U26" s="61" t="n">
+        <f aca="false">IF(20&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V26" s="61" t="n">
+        <f aca="false">IF(21&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W26" s="61" t="n">
+        <f aca="false">IF(22&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X26" s="61" t="n">
+        <f aca="false">IF(23&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y26" s="61" t="n">
+        <f aca="false">IF(24&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z26" s="64" t="n">
+        <f aca="false">SUM(B26:M26)</f>
+        <v>32000</v>
+      </c>
+      <c r="AA26" s="64" t="n">
+        <f aca="false">SUM(N26:Y26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>548</v>
+      </c>
+      <c r="B27" s="61" t="n">
+        <f aca="false">IF(1=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="61" t="n">
+        <f aca="false">IF(2=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="61" t="n">
+        <f aca="false">IF(3=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="61" t="n">
+        <f aca="false">IF(4=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="61" t="n">
+        <f aca="false">IF(5=$B$5,$B$8,0)</f>
+        <v>106250</v>
+      </c>
+      <c r="G27" s="61" t="n">
+        <f aca="false">IF(6=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="61" t="n">
+        <f aca="false">IF(7=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="61" t="n">
+        <f aca="false">IF(8=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="61" t="n">
+        <f aca="false">IF(9=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="61" t="n">
+        <f aca="false">IF(10=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L27" s="61" t="n">
+        <f aca="false">IF(11=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="61" t="n">
+        <f aca="false">IF(12=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N27" s="61" t="n">
+        <f aca="false">IF(13=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O27" s="61" t="n">
+        <f aca="false">IF(14=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P27" s="61" t="n">
+        <f aca="false">IF(15=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="61" t="n">
+        <f aca="false">IF(16=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R27" s="61" t="n">
+        <f aca="false">IF(17=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S27" s="61" t="n">
+        <f aca="false">IF(18=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T27" s="61" t="n">
+        <f aca="false">IF(19=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U27" s="61" t="n">
+        <f aca="false">IF(20=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V27" s="61" t="n">
+        <f aca="false">IF(21=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W27" s="61" t="n">
+        <f aca="false">IF(22=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X27" s="61" t="n">
+        <f aca="false">IF(23=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y27" s="61" t="n">
+        <f aca="false">IF(24=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z27" s="64" t="n">
+        <f aca="false">SUM(B27:M27)</f>
+        <v>106250</v>
+      </c>
+      <c r="AA27" s="64" t="n">
+        <f aca="false">SUM(N27:Y27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>552</v>
+      </c>
+      <c r="B28" s="61" t="n">
+        <f aca="false">IF(AND(1&gt;$B$5,1&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="61" t="n">
+        <f aca="false">IF(AND(2&gt;$B$5,2&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="61" t="n">
+        <f aca="false">IF(AND(3&gt;$B$5,3&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="61" t="n">
+        <f aca="false">IF(AND(4&gt;$B$5,4&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="61" t="n">
+        <f aca="false">IF(AND(5&gt;$B$5,5&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="61" t="n">
+        <f aca="false">IF(AND(6&gt;$B$5,6&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="H28" s="61" t="n">
+        <f aca="false">IF(AND(7&gt;$B$5,7&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="I28" s="61" t="n">
+        <f aca="false">IF(AND(8&gt;$B$5,8&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="J28" s="61" t="n">
+        <f aca="false">IF(AND(9&gt;$B$5,9&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="K28" s="61" t="n">
+        <f aca="false">IF(AND(10&gt;$B$5,10&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="L28" s="61" t="n">
+        <f aca="false">IF(AND(11&gt;$B$5,11&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="M28" s="61" t="n">
+        <f aca="false">IF(AND(12&gt;$B$5,12&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="N28" s="61" t="n">
+        <f aca="false">IF(AND(13&gt;$B$5,13&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="O28" s="61" t="n">
+        <f aca="false">IF(AND(14&gt;$B$5,14&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="P28" s="61" t="n">
+        <f aca="false">IF(AND(15&gt;$B$5,15&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="Q28" s="61" t="n">
+        <f aca="false">IF(AND(16&gt;$B$5,16&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="R28" s="61" t="n">
+        <f aca="false">IF(AND(17&gt;$B$5,17&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="S28" s="61" t="n">
+        <f aca="false">IF(AND(18&gt;$B$5,18&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="T28" s="61" t="n">
+        <f aca="false">IF(AND(19&gt;$B$5,19&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="U28" s="61" t="n">
+        <f aca="false">IF(AND(20&gt;$B$5,20&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="V28" s="61" t="n">
+        <f aca="false">IF(AND(21&gt;$B$5,21&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="W28" s="61" t="n">
+        <f aca="false">IF(AND(22&gt;$B$5,22&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="X28" s="61" t="n">
+        <f aca="false">IF(AND(23&gt;$B$5,23&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>6000</v>
+      </c>
+      <c r="Y28" s="61" t="n">
+        <f aca="false">IF(AND(24&gt;$B$5,24&lt;=$B$5+$B$10),$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z28" s="64" t="n">
+        <f aca="false">SUM(B28:M28)</f>
+        <v>42000</v>
+      </c>
+      <c r="AA28" s="64" t="n">
+        <f aca="false">SUM(N28:Y28)</f>
+        <v>66000</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>553</v>
+      </c>
+      <c r="B29" s="61" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C29" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D29" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E29" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F29" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G29" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H29" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I29" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="J29" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="K29" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="L29" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="M29" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="N29" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="O29" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="P29" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="Q29" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="R29" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="S29" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="T29" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="U29" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="V29" s="61" t="n">
+        <v>17000</v>
+      </c>
+      <c r="W29" s="61" t="n">
+        <v>17000</v>
+      </c>
+      <c r="X29" s="61" t="n">
+        <v>14000</v>
+      </c>
+      <c r="Y29" s="61" t="n">
+        <v>14000</v>
+      </c>
+      <c r="Z29" s="64" t="n">
+        <f aca="false">SUM(B29:M29)</f>
+        <v>104000</v>
+      </c>
+      <c r="AA29" s="64" t="n">
+        <f aca="false">SUM(N29:Y29)</f>
+        <v>188500</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>554</v>
+      </c>
+      <c r="B30" s="64" t="n">
+        <f aca="false">IF(1&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="64" t="n">
+        <f aca="false">IF(2&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="64" t="n">
+        <f aca="false">IF(3&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="64" t="n">
+        <f aca="false">IF(4&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="64" t="n">
+        <f aca="false">IF(5&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="G30" s="64" t="n">
+        <f aca="false">IF(6&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="H30" s="64" t="n">
+        <f aca="false">IF(7&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="I30" s="64" t="n">
+        <f aca="false">IF(8&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="J30" s="64" t="n">
+        <f aca="false">IF(9&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="K30" s="64" t="n">
+        <f aca="false">IF(10&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="L30" s="64" t="n">
+        <f aca="false">IF(11&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="M30" s="64" t="n">
+        <f aca="false">IF(12&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="N30" s="64" t="n">
+        <f aca="false">IF(13&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="O30" s="64" t="n">
+        <f aca="false">IF(14&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="P30" s="64" t="n">
+        <f aca="false">IF(15&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Q30" s="64" t="n">
+        <f aca="false">IF(16&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="R30" s="64" t="n">
+        <f aca="false">IF(17&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="S30" s="64" t="n">
+        <f aca="false">IF(18&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="T30" s="64" t="n">
+        <f aca="false">IF(19&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="U30" s="64" t="n">
+        <f aca="false">IF(20&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="V30" s="64" t="n">
+        <f aca="false">IF(21&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="W30" s="64" t="n">
+        <f aca="false">IF(22&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="X30" s="64" t="n">
+        <f aca="false">IF(23&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Y30" s="64" t="n">
+        <f aca="false">IF(24&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Z30" s="64" t="n">
+        <f aca="false">SUM(B30:M30)</f>
+        <v>-19200</v>
+      </c>
+      <c r="AA30" s="64" t="n">
+        <f aca="false">SUM(N30:Y30)</f>
+        <v>-28800</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="62" t="s">
+        <v>555</v>
+      </c>
+      <c r="B31" s="65" t="n">
+        <f aca="false">B26+B27+B28+B29+B30</f>
+        <v>11500</v>
+      </c>
+      <c r="C31" s="65" t="n">
+        <f aca="false">C26+C27+C28+C29+C30</f>
+        <v>13000</v>
+      </c>
+      <c r="D31" s="65" t="n">
+        <f aca="false">D26+D27+D28+D29+D30</f>
+        <v>13000</v>
+      </c>
+      <c r="E31" s="65" t="n">
+        <f aca="false">E26+E27+E28+E29+E30</f>
+        <v>16000</v>
+      </c>
+      <c r="F31" s="65" t="n">
+        <f aca="false">F26+F27+F28+F29+F30</f>
+        <v>111850</v>
+      </c>
+      <c r="G31" s="65" t="n">
+        <f aca="false">G26+G27+G28+G29+G30</f>
+        <v>11600</v>
+      </c>
+      <c r="H31" s="65" t="n">
+        <f aca="false">H26+H27+H28+H29+H30</f>
+        <v>11600</v>
+      </c>
+      <c r="I31" s="65" t="n">
+        <f aca="false">I26+I27+I28+I29+I30</f>
+        <v>14100</v>
+      </c>
+      <c r="J31" s="65" t="n">
+        <f aca="false">J26+J27+J28+J29+J30</f>
+        <v>14100</v>
+      </c>
+      <c r="K31" s="65" t="n">
+        <f aca="false">K26+K27+K28+K29+K30</f>
+        <v>14100</v>
+      </c>
+      <c r="L31" s="65" t="n">
+        <f aca="false">L26+L27+L28+L29+L30</f>
+        <v>17100</v>
+      </c>
+      <c r="M31" s="65" t="n">
+        <f aca="false">M26+M27+M28+M29+M30</f>
+        <v>17100</v>
+      </c>
+      <c r="N31" s="65" t="n">
+        <f aca="false">N26+N27+N28+N29+N30</f>
+        <v>17100</v>
+      </c>
+      <c r="O31" s="65" t="n">
+        <f aca="false">O26+O27+O28+O29+O30</f>
+        <v>17100</v>
+      </c>
+      <c r="P31" s="65" t="n">
+        <f aca="false">P26+P27+P28+P29+P30</f>
+        <v>17100</v>
+      </c>
+      <c r="Q31" s="65" t="n">
+        <f aca="false">Q26+Q27+Q28+Q29+Q30</f>
+        <v>20100</v>
+      </c>
+      <c r="R31" s="65" t="n">
+        <f aca="false">R26+R27+R28+R29+R30</f>
+        <v>20100</v>
+      </c>
+      <c r="S31" s="65" t="n">
+        <f aca="false">S26+S27+S28+S29+S30</f>
+        <v>20100</v>
+      </c>
+      <c r="T31" s="65" t="n">
+        <f aca="false">T26+T27+T28+T29+T30</f>
+        <v>20100</v>
+      </c>
+      <c r="U31" s="65" t="n">
+        <f aca="false">U26+U27+U28+U29+U30</f>
+        <v>23600</v>
+      </c>
+      <c r="V31" s="65" t="n">
+        <f aca="false">V26+V27+V28+V29+V30</f>
+        <v>20600</v>
+      </c>
+      <c r="W31" s="65" t="n">
+        <f aca="false">W26+W27+W28+W29+W30</f>
+        <v>20600</v>
+      </c>
+      <c r="X31" s="65" t="n">
+        <f aca="false">X26+X27+X28+X29+X30</f>
+        <v>17600</v>
+      </c>
+      <c r="Y31" s="65" t="n">
+        <f aca="false">Y26+Y27+Y28+Y29+Y30</f>
+        <v>11600</v>
+      </c>
+      <c r="Z31" s="65" t="n">
+        <f aca="false">SUM(B31:M31)</f>
+        <v>265050</v>
+      </c>
+      <c r="AA31" s="65" t="n">
+        <f aca="false">SUM(N31:Y31)</f>
+        <v>225700</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="50" t="s">
+        <v>556</v>
+      </c>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="50"/>
+      <c r="G33" s="50"/>
+      <c r="H33" s="50"/>
+      <c r="I33" s="50"/>
+      <c r="J33" s="50"/>
+      <c r="K33" s="50"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="50"/>
+      <c r="O33" s="50"/>
+      <c r="P33" s="50"/>
+      <c r="Q33" s="50"/>
+      <c r="R33" s="50"/>
+      <c r="S33" s="50"/>
+      <c r="T33" s="50"/>
+      <c r="U33" s="50"/>
+      <c r="V33" s="50"/>
+      <c r="W33" s="50"/>
+      <c r="X33" s="50"/>
+      <c r="Y33" s="50"/>
+      <c r="Z33" s="50"/>
+      <c r="AA33" s="50"/>
+      <c r="AB33" s="50"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>557</v>
+      </c>
+      <c r="B34" s="61" t="n">
+        <f aca="false">IF(1&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="C34" s="61" t="n">
+        <f aca="false">IF(2&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="D34" s="61" t="n">
+        <f aca="false">IF(3&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="E34" s="61" t="n">
+        <f aca="false">IF(4&lt;$B$5,8000,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="F34" s="61" t="n">
+        <f aca="false">IF(5&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="61" t="n">
+        <f aca="false">IF(6&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="61" t="n">
+        <f aca="false">IF(7&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="61" t="n">
+        <f aca="false">IF(8&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="61" t="n">
+        <f aca="false">IF(9&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K34" s="61" t="n">
+        <f aca="false">IF(10&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L34" s="61" t="n">
+        <f aca="false">IF(11&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M34" s="61" t="n">
+        <f aca="false">IF(12&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N34" s="61" t="n">
+        <f aca="false">IF(13&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O34" s="61" t="n">
+        <f aca="false">IF(14&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="61" t="n">
+        <f aca="false">IF(15&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="61" t="n">
+        <f aca="false">IF(16&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R34" s="61" t="n">
+        <f aca="false">IF(17&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S34" s="61" t="n">
+        <f aca="false">IF(18&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T34" s="61" t="n">
+        <f aca="false">IF(19&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U34" s="61" t="n">
+        <f aca="false">IF(20&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V34" s="61" t="n">
+        <f aca="false">IF(21&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W34" s="61" t="n">
+        <f aca="false">IF(22&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X34" s="61" t="n">
+        <f aca="false">IF(23&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y34" s="61" t="n">
+        <f aca="false">IF(24&lt;$B$5,8000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z34" s="64" t="n">
+        <f aca="false">SUM(B34:M34)</f>
+        <v>32000</v>
+      </c>
+      <c r="AA34" s="64" t="n">
+        <f aca="false">SUM(N34:Y34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>548</v>
+      </c>
+      <c r="B35" s="61" t="n">
+        <f aca="false">IF(1=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="61" t="n">
+        <f aca="false">IF(2=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="61" t="n">
+        <f aca="false">IF(3=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="61" t="n">
+        <f aca="false">IF(4=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="61" t="n">
+        <f aca="false">IF(5=$B$5,$B$8,0)</f>
+        <v>106250</v>
+      </c>
+      <c r="G35" s="61" t="n">
+        <f aca="false">IF(6=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="61" t="n">
+        <f aca="false">IF(7=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="61" t="n">
+        <f aca="false">IF(8=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="61" t="n">
+        <f aca="false">IF(9=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K35" s="61" t="n">
+        <f aca="false">IF(10=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L35" s="61" t="n">
+        <f aca="false">IF(11=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M35" s="61" t="n">
+        <f aca="false">IF(12=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N35" s="61" t="n">
+        <f aca="false">IF(13=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O35" s="61" t="n">
+        <f aca="false">IF(14=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P35" s="61" t="n">
+        <f aca="false">IF(15=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="61" t="n">
+        <f aca="false">IF(16=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R35" s="61" t="n">
+        <f aca="false">IF(17=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="S35" s="61" t="n">
+        <f aca="false">IF(18=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T35" s="61" t="n">
+        <f aca="false">IF(19=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="U35" s="61" t="n">
+        <f aca="false">IF(20=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="V35" s="61" t="n">
+        <f aca="false">IF(21=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W35" s="61" t="n">
+        <f aca="false">IF(22=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X35" s="61" t="n">
+        <f aca="false">IF(23=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y35" s="61" t="n">
+        <f aca="false">IF(24=$B$5,$B$8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z35" s="64" t="n">
+        <f aca="false">SUM(B35:M35)</f>
+        <v>106250</v>
+      </c>
+      <c r="AA35" s="64" t="n">
+        <f aca="false">SUM(N35:Y35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>558</v>
+      </c>
+      <c r="B36" s="61" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C36" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D36" s="61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E36" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F36" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G36" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H36" s="61" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I36" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="J36" s="61" t="n">
+        <v>10500</v>
+      </c>
+      <c r="K36" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="L36" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="M36" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="N36" s="61" t="n">
+        <v>13500</v>
+      </c>
+      <c r="O36" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="P36" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="Q36" s="61" t="n">
+        <v>16500</v>
+      </c>
+      <c r="R36" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="S36" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="T36" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="U36" s="61" t="n">
+        <v>23000</v>
+      </c>
+      <c r="V36" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="W36" s="61" t="n">
+        <v>20000</v>
+      </c>
+      <c r="X36" s="61" t="n">
+        <v>20500</v>
+      </c>
+      <c r="Y36" s="61" t="n">
+        <v>20500</v>
+      </c>
+      <c r="Z36" s="64" t="n">
+        <f aca="false">SUM(B36:M36)</f>
+        <v>107000</v>
+      </c>
+      <c r="AA36" s="64" t="n">
+        <f aca="false">SUM(N36:Y36)</f>
+        <v>227000</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>554</v>
+      </c>
+      <c r="B37" s="64" t="n">
+        <f aca="false">IF(1&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="64" t="n">
+        <f aca="false">IF(2&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="64" t="n">
+        <f aca="false">IF(3&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="64" t="n">
+        <f aca="false">IF(4&gt;=$B$11,-$B$12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="64" t="n">
+        <f aca="false">IF(5&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="G37" s="64" t="n">
+        <f aca="false">IF(6&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="H37" s="64" t="n">
+        <f aca="false">IF(7&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="I37" s="64" t="n">
+        <f aca="false">IF(8&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="J37" s="64" t="n">
+        <f aca="false">IF(9&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="K37" s="64" t="n">
+        <f aca="false">IF(10&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="L37" s="64" t="n">
+        <f aca="false">IF(11&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="M37" s="64" t="n">
+        <f aca="false">IF(12&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="N37" s="64" t="n">
+        <f aca="false">IF(13&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="O37" s="64" t="n">
+        <f aca="false">IF(14&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="P37" s="64" t="n">
+        <f aca="false">IF(15&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Q37" s="64" t="n">
+        <f aca="false">IF(16&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="R37" s="64" t="n">
+        <f aca="false">IF(17&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="S37" s="64" t="n">
+        <f aca="false">IF(18&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="T37" s="64" t="n">
+        <f aca="false">IF(19&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="U37" s="64" t="n">
+        <f aca="false">IF(20&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="V37" s="64" t="n">
+        <f aca="false">IF(21&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="W37" s="64" t="n">
+        <f aca="false">IF(22&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="X37" s="64" t="n">
+        <f aca="false">IF(23&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Y37" s="64" t="n">
+        <f aca="false">IF(24&gt;=$B$11,-$B$12,0)</f>
+        <v>-2400</v>
+      </c>
+      <c r="Z37" s="64" t="n">
+        <f aca="false">SUM(B37:M37)</f>
+        <v>-19200</v>
+      </c>
+      <c r="AA37" s="64" t="n">
+        <f aca="false">SUM(N37:Y37)</f>
+        <v>-28800</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="62" t="s">
+        <v>559</v>
+      </c>
+      <c r="B38" s="65" t="n">
+        <f aca="false">B34+B35+B36+B37</f>
+        <v>11500</v>
+      </c>
+      <c r="C38" s="65" t="n">
+        <f aca="false">C34+C35+C36+C37</f>
+        <v>13000</v>
+      </c>
+      <c r="D38" s="65" t="n">
+        <f aca="false">D34+D35+D36+D37</f>
+        <v>13000</v>
+      </c>
+      <c r="E38" s="65" t="n">
+        <f aca="false">E34+E35+E36+E37</f>
+        <v>16000</v>
+      </c>
+      <c r="F38" s="65" t="n">
+        <f aca="false">F34+F35+F36+F37</f>
+        <v>111850</v>
+      </c>
+      <c r="G38" s="65" t="n">
+        <f aca="false">G34+G35+G36+G37</f>
+        <v>5600</v>
+      </c>
+      <c r="H38" s="65" t="n">
+        <f aca="false">H34+H35+H36+H37</f>
+        <v>5600</v>
+      </c>
+      <c r="I38" s="65" t="n">
+        <f aca="false">I34+I35+I36+I37</f>
+        <v>8100</v>
+      </c>
+      <c r="J38" s="65" t="n">
+        <f aca="false">J34+J35+J36+J37</f>
+        <v>8100</v>
+      </c>
+      <c r="K38" s="65" t="n">
+        <f aca="false">K34+K35+K36+K37</f>
+        <v>11100</v>
+      </c>
+      <c r="L38" s="65" t="n">
+        <f aca="false">L34+L35+L36+L37</f>
+        <v>11100</v>
+      </c>
+      <c r="M38" s="65" t="n">
+        <f aca="false">M34+M35+M36+M37</f>
+        <v>11100</v>
+      </c>
+      <c r="N38" s="65" t="n">
+        <f aca="false">N34+N35+N36+N37</f>
+        <v>11100</v>
+      </c>
+      <c r="O38" s="65" t="n">
+        <f aca="false">O34+O35+O36+O37</f>
+        <v>14100</v>
+      </c>
+      <c r="P38" s="65" t="n">
+        <f aca="false">P34+P35+P36+P37</f>
+        <v>14100</v>
+      </c>
+      <c r="Q38" s="65" t="n">
+        <f aca="false">Q34+Q35+Q36+Q37</f>
+        <v>14100</v>
+      </c>
+      <c r="R38" s="65" t="n">
+        <f aca="false">R34+R35+R36+R37</f>
+        <v>17600</v>
+      </c>
+      <c r="S38" s="65" t="n">
+        <f aca="false">S34+S35+S36+S37</f>
+        <v>17600</v>
+      </c>
+      <c r="T38" s="65" t="n">
+        <f aca="false">T34+T35+T36+T37</f>
+        <v>17600</v>
+      </c>
+      <c r="U38" s="65" t="n">
+        <f aca="false">U34+U35+U36+U37</f>
+        <v>20600</v>
+      </c>
+      <c r="V38" s="65" t="n">
+        <f aca="false">V34+V35+V36+V37</f>
+        <v>17600</v>
+      </c>
+      <c r="W38" s="65" t="n">
+        <f aca="false">W34+W35+W36+W37</f>
+        <v>17600</v>
+      </c>
+      <c r="X38" s="65" t="n">
+        <f aca="false">X34+X35+X36+X37</f>
+        <v>18100</v>
+      </c>
+      <c r="Y38" s="65" t="n">
+        <f aca="false">Y34+Y35+Y36+Y37</f>
+        <v>18100</v>
+      </c>
+      <c r="Z38" s="65" t="n">
+        <f aca="false">SUM(B38:M38)</f>
+        <v>226050</v>
+      </c>
+      <c r="AA38" s="65" t="n">
+        <f aca="false">SUM(N38:Y38)</f>
+        <v>198200</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="50" t="s">
+        <v>560</v>
+      </c>
+      <c r="B40" s="50"/>
+      <c r="C40" s="50"/>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="50"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" s="30" t="s">
+        <v>561</v>
+      </c>
+      <c r="C41" s="30" t="s">
+        <v>562</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>563</v>
+      </c>
+      <c r="E41" s="30" t="s">
+        <v>564</v>
+      </c>
+      <c r="F41" s="30" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>565</v>
+      </c>
+      <c r="B42" s="66" t="n">
+        <f aca="false">Z23</f>
+        <v>300250</v>
+      </c>
+      <c r="C42" s="66" t="n">
+        <f aca="false">AA23</f>
+        <v>255000</v>
+      </c>
+      <c r="D42" s="66" t="n">
+        <f aca="false">B42+C42</f>
+        <v>555250</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>566</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="67" t="s">
+        <v>568</v>
+      </c>
+      <c r="B43" s="68" t="n">
+        <f aca="false">Z31</f>
+        <v>265050</v>
+      </c>
+      <c r="C43" s="68" t="n">
+        <f aca="false">AA31</f>
+        <v>225700</v>
+      </c>
+      <c r="D43" s="68" t="n">
+        <f aca="false">B43+C43</f>
+        <v>490750</v>
+      </c>
+      <c r="E43" s="67" t="s">
+        <v>569</v>
+      </c>
+      <c r="F43" s="67" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>571</v>
+      </c>
+      <c r="B44" s="66" t="n">
+        <f aca="false">Z38</f>
+        <v>226050</v>
+      </c>
+      <c r="C44" s="66" t="n">
+        <f aca="false">AA38</f>
+        <v>198200</v>
+      </c>
+      <c r="D44" s="66" t="n">
+        <f aca="false">B44+C44</f>
+        <v>424250</v>
+      </c>
+      <c r="E44" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="50" t="s">
+        <v>574</v>
+      </c>
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+      <c r="E46" s="50"/>
+      <c r="F46" s="50"/>
+      <c r="G46" s="50"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="s">
+        <v>575</v>
+      </c>
+      <c r="B47" s="69" t="n">
+        <f aca="false">B15</f>
+        <v>21</v>
+      </c>
+      <c r="C47" s="52" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
+        <v>577</v>
+      </c>
+      <c r="B48" s="69" t="n">
+        <f aca="false">3*18</f>
+        <v>54</v>
+      </c>
+      <c r="C48" s="52" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>579</v>
+      </c>
+      <c r="B49" s="69" t="n">
+        <f aca="false">173/12</f>
+        <v>14.4166666666667</v>
+      </c>
+      <c r="C49" s="52" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
+        <v>581</v>
+      </c>
+      <c r="B50" s="69" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="52" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="62" t="s">
+        <v>583</v>
+      </c>
+      <c r="B51" s="70" t="n">
+        <f aca="false">B47+B48+B49+B50</f>
+        <v>119.416666666667</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>584</v>
+      </c>
+      <c r="B52" s="69" t="n">
+        <v>180</v>
+      </c>
+      <c r="C52" s="52" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="62" t="s">
+        <v>586</v>
+      </c>
+      <c r="B53" s="71" t="n">
+        <f aca="false">B52-B51</f>
+        <v>60.5833333333333</v>
+      </c>
+      <c r="C53" s="52" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="B55" s="50"/>
+      <c r="C55" s="50"/>
+      <c r="D55" s="50"/>
+      <c r="E55" s="50"/>
+      <c r="F55" s="50"/>
+      <c r="G55" s="50"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="27" t="s">
+        <v>589</v>
+      </c>
+      <c r="B56" s="27"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="27"/>
+      <c r="H56" s="27"/>
+      <c r="I56" s="27"/>
+      <c r="J56" s="27"/>
+      <c r="K56" s="27"/>
+      <c r="L56" s="27"/>
+      <c r="M56" s="27"/>
+      <c r="N56" s="27"/>
+      <c r="O56" s="27"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="27" t="s">
+        <v>590</v>
+      </c>
+      <c r="B57" s="27"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="27"/>
+      <c r="H57" s="27"/>
+      <c r="I57" s="27"/>
+      <c r="J57" s="27"/>
+      <c r="K57" s="27"/>
+      <c r="L57" s="27"/>
+      <c r="M57" s="27"/>
+      <c r="N57" s="27"/>
+      <c r="O57" s="27"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="27" t="s">
+        <v>591</v>
+      </c>
+      <c r="B58" s="27"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="27"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="27"/>
+      <c r="H58" s="27"/>
+      <c r="I58" s="27"/>
+      <c r="J58" s="27"/>
+      <c r="K58" s="27"/>
+      <c r="L58" s="27"/>
+      <c r="M58" s="27"/>
+      <c r="N58" s="27"/>
+      <c r="O58" s="27"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="27" t="s">
+        <v>592</v>
+      </c>
+      <c r="B59" s="27"/>
+      <c r="C59" s="27"/>
+      <c r="D59" s="27"/>
+      <c r="E59" s="27"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="27"/>
+      <c r="H59" s="27"/>
+      <c r="I59" s="27"/>
+      <c r="J59" s="27"/>
+      <c r="K59" s="27"/>
+      <c r="L59" s="27"/>
+      <c r="M59" s="27"/>
+      <c r="N59" s="27"/>
+      <c r="O59" s="27"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="27" t="s">
+        <v>593</v>
+      </c>
+      <c r="B60" s="27"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="F60" s="27"/>
+      <c r="G60" s="27"/>
+      <c r="H60" s="27"/>
+      <c r="I60" s="27"/>
+      <c r="J60" s="27"/>
+      <c r="K60" s="27"/>
+      <c r="L60" s="27"/>
+      <c r="M60" s="27"/>
+      <c r="N60" s="27"/>
+      <c r="O60" s="27"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="27" t="s">
+        <v>594</v>
+      </c>
+      <c r="B61" s="27"/>
+      <c r="C61" s="27"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="27"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="27"/>
+      <c r="H61" s="27"/>
+      <c r="I61" s="27"/>
+      <c r="J61" s="27"/>
+      <c r="K61" s="27"/>
+      <c r="L61" s="27"/>
+      <c r="M61" s="27"/>
+      <c r="N61" s="27"/>
+      <c r="O61" s="27"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="27" t="s">
+        <v>595</v>
+      </c>
+      <c r="B62" s="27"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27"/>
+      <c r="E62" s="27"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="27"/>
+      <c r="H62" s="27"/>
+      <c r="I62" s="27"/>
+      <c r="J62" s="27"/>
+      <c r="K62" s="27"/>
+      <c r="L62" s="27"/>
+      <c r="M62" s="27"/>
+      <c r="N62" s="27"/>
+      <c r="O62" s="27"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="27" t="s">
+        <v>596</v>
+      </c>
+      <c r="B63" s="27"/>
+      <c r="C63" s="27"/>
+      <c r="D63" s="27"/>
+      <c r="E63" s="27"/>
+      <c r="F63" s="27"/>
+      <c r="G63" s="27"/>
+      <c r="H63" s="27"/>
+      <c r="I63" s="27"/>
+      <c r="J63" s="27"/>
+      <c r="K63" s="27"/>
+      <c r="L63" s="27"/>
+      <c r="M63" s="27"/>
+      <c r="N63" s="27"/>
+      <c r="O63" s="27"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="27" t="s">
+        <v>597</v>
+      </c>
+      <c r="B64" s="27"/>
+      <c r="C64" s="27"/>
+      <c r="D64" s="27"/>
+      <c r="E64" s="27"/>
+      <c r="F64" s="27"/>
+      <c r="G64" s="27"/>
+      <c r="H64" s="27"/>
+      <c r="I64" s="27"/>
+      <c r="J64" s="27"/>
+      <c r="K64" s="27"/>
+      <c r="L64" s="27"/>
+      <c r="M64" s="27"/>
+      <c r="N64" s="27"/>
+      <c r="O64" s="27"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A1:AA1"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A19:AB19"/>
+    <mergeCell ref="A25:AB25"/>
+    <mergeCell ref="A33:AB33"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A56:O56"/>
+    <mergeCell ref="A57:O57"/>
+    <mergeCell ref="A58:O58"/>
+    <mergeCell ref="A59:O59"/>
+    <mergeCell ref="A60:O60"/>
+    <mergeCell ref="A61:O61"/>
+    <mergeCell ref="A62:O62"/>
+    <mergeCell ref="A63:O63"/>
+    <mergeCell ref="A64:O64"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
vault backup: 2026-05-30 23:30:28
</commit_message>
<xml_diff>
--- a/income_forecaster.xlsx
+++ b/income_forecaster.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="606">
   <si>
     <t xml:space="preserve">Income Forecaster — Chance Peare</t>
   </si>
@@ -174,7 +174,7 @@
     <t xml:space="preserve">Health insurance (paycheck)</t>
   </si>
   <si>
-    <t xml:space="preserve">Midpoint of $200–600 range.</t>
+    <t xml:space="preserve">Currently $400 (Skyright payroll). Post-sale (Scenarios B/C): $600 health sharing ministry, $7.2K/yr — saves $15-23K vs ACA but NOT insurance.</t>
   </si>
   <si>
     <t xml:space="preserve">Auto loan payment</t>
@@ -1614,16 +1614,16 @@
     <t xml:space="preserve">Equity payment (gross)</t>
   </si>
   <si>
-    <t xml:space="preserve">5% stake. Mid-low of $100-200K range.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LTCG tax rate (federal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15% MFJ for AGI &lt; $583K. Assumes &gt;1-yr holding.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equity payment (net of tax)</t>
+    <t xml:space="preserve">5% phantom equity. Working equity, no basis. Taxable as ordinary income.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective tax on equity (ordinary income + FICA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phantom/ghost equity = W2 wages. 22-24% federal + 7.65% FICA at this income.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity payment (net of tax &amp; FICA)</t>
   </si>
   <si>
     <t xml:space="preserve">Net cash to bank.</t>
@@ -1764,7 +1764,7 @@
     <t xml:space="preserve">Reduced from 35 to ~21 hrs/mo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Other retainer hrs/mo (3 retainers × 18 hrs)</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">Active tier ~18 hrs/mo each.</t>
@@ -1797,34 +1797,58 @@
     <t xml:space="preserve">Positive = fits. Negative = need to drop a retainer or hire more.</t>
   </si>
   <si>
-    <t xml:space="preserve">STRATEGIC NOTES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Equity tax treatment: assumes LTCG (&gt;1-yr holding). Federal 15% MFJ at AGI &lt;$583K. Verify cost basis with CPA — could be lower than gross if exercised options.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Scenario B (Skyright as Embedded) requires the BUYER to want this arrangement. Most likely if buyer is owner-operator or strategic acquirer who values continuity. PE buyers typically install own ops team — Scenario B unlikely with PE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Skyright Embedded duration (18 months default) is aggressive. Reality: transition retainers often end in 6-12 months once new ops team is in place. Edit Assumptions B10 to test 12-mo case.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• VA hired at sale month to absorb Skyright admin/operational work. Make automations + ServiceTitan integrations + report automation = the 40% time savings on Skyright retainer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• In Scenario B, Skyright becomes both an income source AND your capacity sink. If they need 21 hrs/mo, you only have ~159 hrs/mo for everything else. Tight.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Scenario C buys runway with equity but requires faster client acquisition to compensate for lost Skyright income. Aggressive growth path assumes 6 active retainers by end Y2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Equity payment goes into Mercury business account if treated as business income, OR personal if treated as capital gains on personal investment. Most likely the latter (personal LTCG). Confirm with CPA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Health insurance: Scenario A keeps Skyright/NewCo employer coverage. B and C trigger ACA ($1,500-2,500/mo family of 6) starting sale month. NOT modeled here — add $18-30K/yr cost to B and C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Tax estimate on Y1 numbers gets complicated: W2 portion withheld, 1099 portion + equity (LTCG) require separate quarterly payments. Cleanup at year-end could be a $10K+ surprise either direction.</t>
+    <t xml:space="preserve">STRATEGIC NOTES (UPDATED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Equity is PHANTOM/GHOST equity — taxed as W2 ordinary income + FICA. ~30% effective rate at this income. Net = ~$87.5K on $125K gross. NOT LTCG.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Confirm with CPA whether equity payment can use §409A structuring to defer or restructure timing. Could push payment to following tax year if you want to manage AGI for QBI / ACA / etc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Health coverage: Health sharing ministry at $600/mo (~$7,200/yr) for Scenarios B and C. Saves $15-23K vs ACA — but health sharing is NOT insurance, has limits, may not cover pre-existing conditions. Material risk for family of 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Buyer is likely strategic or owner-operator (per discussion). Scenario B (Skyright as Embedded) is REALISTIC, not aspirational. Now actively negotiate the retainer arrangement with current owner BEFORE sale — write it into sale documents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Push for premium Embedded $8-10K/mo for first 12 months, stepping down to $6K thereafter. Current owner can include this as a transition condition in the sale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• You are already building JobNimbus estimating tools + office automation at Skyright. CRITICAL — clarify IP ownership NOW. Workflows in JobNimbus stay with Skyright (their seat). Make/Zapier automations under your accounts could be portable. Best path: document everything as Skyright IP, license-back through retainer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Automation work you're doing reduces Skyright Embedded hours needed post-sale (already estimated at 40% reduction). Good — but means the buyer values this automation portfolio. Don't under-price the retainer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• If buyer turns out to be PE (unlikely per your read but possible), Scenario B falls apart — PE installs own ops team. Plan B fallback should be Scenario C (clean exit on equity runway).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Year 1 tax with equity = COMPLICATED. W2 income (Skyright $96K + equity $125K = $221K) + 1099 ($85.5K) = $306K gross. Marginal rate hits 24%. Effective rate ~22-25%. Quarterly estimated payments need to scale up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cash inflow concentration: home sale ($95K July) + equity ($87.5K Oct) + retainer income = ~$200K of one-time cash in Q3-Q4 2026. Deploy intentionally: debt payoff first, emergency fund second, business reserves third, retirement contribution fourth.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WEIGHTED SCENARIO (planning baseline)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability A (Stay at NewCo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability B (Skyright as Embedded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability C (Clean exit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted Y1 Gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted Y2 Gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted 24-mo Total</t>
   </si>
 </sst>
 </file>
@@ -1840,8 +1864,8 @@
     <numFmt numFmtId="169" formatCode="0.00%"/>
     <numFmt numFmtId="170" formatCode="0.0000"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0"/>
-    <numFmt numFmtId="173" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="172" formatCode="0%"/>
+    <numFmt numFmtId="173" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -2024,7 +2048,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2217,11 +2241,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2229,47 +2273,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="172" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2277,39 +2281,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="173" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4584,215 +4556,215 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB64"/>
+  <dimension ref="A1:AB82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="7" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="48" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
-      <c r="W1" s="48"/>
-      <c r="X1" s="48"/>
-      <c r="Y1" s="48"/>
-      <c r="Z1" s="48"/>
-      <c r="AA1" s="48"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="49" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>522</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="49"/>
-      <c r="R2" s="49"/>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="49"/>
-      <c r="V2" s="49"/>
-      <c r="W2" s="49"/>
-      <c r="X2" s="49"/>
-      <c r="Y2" s="49"/>
-      <c r="Z2" s="49"/>
-      <c r="AA2" s="49"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="50" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="B5" s="51" t="n">
+      <c r="B5" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="6" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="B6" s="53" t="n">
+      <c r="B6" s="15" t="n">
         <v>125000</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="6" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="B7" s="54" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C7" s="52" t="s">
+      <c r="B7" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="B8" s="55" t="n">
+      <c r="B8" s="48" t="n">
         <f aca="false">B6*(1-B7)</f>
-        <v>106250</v>
-      </c>
-      <c r="C8" s="52" t="s">
+        <v>87500</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="B9" s="56" t="n">
+      <c r="B9" s="14" t="n">
         <v>6000</v>
       </c>
-      <c r="C9" s="52" t="s">
+      <c r="C9" s="6" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="B10" s="51" t="n">
+      <c r="B10" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="C10" s="52" t="s">
+      <c r="C10" s="6" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="B11" s="51" t="n">
+      <c r="B11" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="6" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="B12" s="56" t="n">
+      <c r="B12" s="14" t="n">
         <v>2400</v>
       </c>
-      <c r="C12" s="52" t="s">
+      <c r="C12" s="6" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="B13" s="57" t="n">
+      <c r="B13" s="36" t="n">
         <v>0.4</v>
       </c>
-      <c r="C13" s="52" t="s">
+      <c r="C13" s="6" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="B14" s="58" t="n">
+      <c r="B14" s="33" t="n">
         <v>35</v>
       </c>
-      <c r="C14" s="52" t="s">
+      <c r="C14" s="6" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="B15" s="59" t="n">
+      <c r="B15" s="45" t="n">
         <f aca="false">B14*(1-B13)</f>
         <v>21</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="6" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="60" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="40" t="s">
         <v>192</v>
       </c>
       <c r="B17" s="30" t="s">
@@ -4867,1660 +4839,1660 @@
       <c r="Y17" s="30" t="s">
         <v>332</v>
       </c>
-      <c r="Z17" s="60" t="s">
+      <c r="Z17" s="40" t="s">
         <v>345</v>
       </c>
-      <c r="AA17" s="60" t="s">
+      <c r="AA17" s="40" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="50" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>546</v>
       </c>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="50"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="Q19" s="50"/>
-      <c r="R19" s="50"/>
-      <c r="S19" s="50"/>
-      <c r="T19" s="50"/>
-      <c r="U19" s="50"/>
-      <c r="V19" s="50"/>
-      <c r="W19" s="50"/>
-      <c r="X19" s="50"/>
-      <c r="Y19" s="50"/>
-      <c r="Z19" s="50"/>
-      <c r="AA19" s="50"/>
-      <c r="AB19" s="50"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="4"/>
+      <c r="X19" s="4"/>
+      <c r="Y19" s="4"/>
+      <c r="Z19" s="4"/>
+      <c r="AA19" s="4"/>
+      <c r="AB19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="B20" s="61" t="n">
+      <c r="B20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="C20" s="61" t="n">
+      <c r="C20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="D20" s="61" t="n">
+      <c r="D20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="E20" s="61" t="n">
+      <c r="E20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="F20" s="61" t="n">
+      <c r="F20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="G20" s="61" t="n">
+      <c r="G20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="H20" s="61" t="n">
+      <c r="H20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="I20" s="61" t="n">
+      <c r="I20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="J20" s="61" t="n">
+      <c r="J20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="K20" s="61" t="n">
+      <c r="K20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="L20" s="61" t="n">
+      <c r="L20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="M20" s="61" t="n">
+      <c r="M20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="N20" s="61" t="n">
+      <c r="N20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="O20" s="61" t="n">
+      <c r="O20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="P20" s="61" t="n">
+      <c r="P20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="Q20" s="61" t="n">
+      <c r="Q20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="R20" s="61" t="n">
+      <c r="R20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="S20" s="61" t="n">
+      <c r="S20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="T20" s="61" t="n">
+      <c r="T20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="U20" s="61" t="n">
+      <c r="U20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="V20" s="61" t="n">
+      <c r="V20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="W20" s="61" t="n">
+      <c r="W20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="X20" s="61" t="n">
+      <c r="X20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="Y20" s="61" t="n">
+      <c r="Y20" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="Z20" s="55" t="n">
+      <c r="Z20" s="48" t="n">
         <f aca="false">SUM(B20:M20)</f>
         <v>96000</v>
       </c>
-      <c r="AA20" s="55" t="n">
+      <c r="AA20" s="48" t="n">
         <f aca="false">SUM(N20:Y20)</f>
         <v>96000</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B21" s="61" t="n">
+      <c r="B21" s="38" t="n">
         <f aca="false">IF(1=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="C21" s="61" t="n">
+      <c r="C21" s="38" t="n">
         <f aca="false">IF(2=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="61" t="n">
+      <c r="D21" s="38" t="n">
         <f aca="false">IF(3=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="61" t="n">
+      <c r="E21" s="38" t="n">
         <f aca="false">IF(4=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="61" t="n">
+      <c r="F21" s="38" t="n">
         <f aca="false">IF(5=$B$5,$B$8,0)</f>
-        <v>106250</v>
-      </c>
-      <c r="G21" s="61" t="n">
+        <v>87500</v>
+      </c>
+      <c r="G21" s="38" t="n">
         <f aca="false">IF(6=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="H21" s="61" t="n">
+      <c r="H21" s="38" t="n">
         <f aca="false">IF(7=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="I21" s="61" t="n">
+      <c r="I21" s="38" t="n">
         <f aca="false">IF(8=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="61" t="n">
+      <c r="J21" s="38" t="n">
         <f aca="false">IF(9=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="61" t="n">
+      <c r="K21" s="38" t="n">
         <f aca="false">IF(10=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="61" t="n">
+      <c r="L21" s="38" t="n">
         <f aca="false">IF(11=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="M21" s="61" t="n">
+      <c r="M21" s="38" t="n">
         <f aca="false">IF(12=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="N21" s="61" t="n">
+      <c r="N21" s="38" t="n">
         <f aca="false">IF(13=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="O21" s="61" t="n">
+      <c r="O21" s="38" t="n">
         <f aca="false">IF(14=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="P21" s="61" t="n">
+      <c r="P21" s="38" t="n">
         <f aca="false">IF(15=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Q21" s="61" t="n">
+      <c r="Q21" s="38" t="n">
         <f aca="false">IF(16=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="R21" s="61" t="n">
+      <c r="R21" s="38" t="n">
         <f aca="false">IF(17=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="S21" s="61" t="n">
+      <c r="S21" s="38" t="n">
         <f aca="false">IF(18=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="T21" s="61" t="n">
+      <c r="T21" s="38" t="n">
         <f aca="false">IF(19=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="U21" s="61" t="n">
+      <c r="U21" s="38" t="n">
         <f aca="false">IF(20=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="V21" s="61" t="n">
+      <c r="V21" s="38" t="n">
         <f aca="false">IF(21=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="W21" s="61" t="n">
+      <c r="W21" s="38" t="n">
         <f aca="false">IF(22=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="X21" s="61" t="n">
+      <c r="X21" s="38" t="n">
         <f aca="false">IF(23=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Y21" s="61" t="n">
+      <c r="Y21" s="38" t="n">
         <f aca="false">IF(24=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Z21" s="55" t="n">
+      <c r="Z21" s="48" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>106250</v>
-      </c>
-      <c r="AA21" s="55" t="n">
+        <v>87500</v>
+      </c>
+      <c r="AA21" s="48" t="n">
         <f aca="false">SUM(N21:Y21)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="B22" s="61" t="n">
+      <c r="B22" s="38" t="n">
         <v>3500</v>
       </c>
-      <c r="C22" s="61" t="n">
+      <c r="C22" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="D22" s="61" t="n">
+      <c r="D22" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="E22" s="61" t="n">
+      <c r="E22" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="F22" s="61" t="n">
+      <c r="F22" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="G22" s="61" t="n">
+      <c r="G22" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="H22" s="61" t="n">
+      <c r="H22" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="I22" s="61" t="n">
+      <c r="I22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="J22" s="61" t="n">
+      <c r="J22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="K22" s="61" t="n">
+      <c r="K22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="L22" s="61" t="n">
+      <c r="L22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="M22" s="61" t="n">
+      <c r="M22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="N22" s="61" t="n">
+      <c r="N22" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="O22" s="61" t="n">
+      <c r="O22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="P22" s="61" t="n">
+      <c r="P22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="Q22" s="61" t="n">
+      <c r="Q22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="R22" s="61" t="n">
+      <c r="R22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="S22" s="61" t="n">
+      <c r="S22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="T22" s="61" t="n">
+      <c r="T22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="U22" s="61" t="n">
+      <c r="U22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="V22" s="61" t="n">
+      <c r="V22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="W22" s="61" t="n">
+      <c r="W22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="X22" s="61" t="n">
+      <c r="X22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="Y22" s="61" t="n">
+      <c r="Y22" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="Z22" s="55" t="n">
+      <c r="Z22" s="48" t="n">
         <f aca="false">SUM(B22:M22)</f>
         <v>98000</v>
       </c>
-      <c r="AA22" s="55" t="n">
+      <c r="AA22" s="48" t="n">
         <f aca="false">SUM(N22:Y22)</f>
         <v>159000</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="62" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B23" s="63" t="n">
+      <c r="B23" s="49" t="n">
         <f aca="false">B20+B21+B22</f>
         <v>11500</v>
       </c>
-      <c r="C23" s="63" t="n">
+      <c r="C23" s="49" t="n">
         <f aca="false">C20+C21+C22</f>
         <v>13000</v>
       </c>
-      <c r="D23" s="63" t="n">
+      <c r="D23" s="49" t="n">
         <f aca="false">D20+D21+D22</f>
         <v>13000</v>
       </c>
-      <c r="E23" s="63" t="n">
+      <c r="E23" s="49" t="n">
         <f aca="false">E20+E21+E22</f>
         <v>16000</v>
       </c>
-      <c r="F23" s="63" t="n">
+      <c r="F23" s="49" t="n">
         <f aca="false">F20+F21+F22</f>
-        <v>122250</v>
-      </c>
-      <c r="G23" s="63" t="n">
+        <v>103500</v>
+      </c>
+      <c r="G23" s="49" t="n">
         <f aca="false">G20+G21+G22</f>
         <v>16000</v>
       </c>
-      <c r="H23" s="63" t="n">
+      <c r="H23" s="49" t="n">
         <f aca="false">H20+H21+H22</f>
         <v>16000</v>
       </c>
-      <c r="I23" s="63" t="n">
+      <c r="I23" s="49" t="n">
         <f aca="false">I20+I21+I22</f>
         <v>18500</v>
       </c>
-      <c r="J23" s="63" t="n">
+      <c r="J23" s="49" t="n">
         <f aca="false">J20+J21+J22</f>
         <v>18500</v>
       </c>
-      <c r="K23" s="63" t="n">
+      <c r="K23" s="49" t="n">
         <f aca="false">K20+K21+K22</f>
         <v>18500</v>
       </c>
-      <c r="L23" s="63" t="n">
+      <c r="L23" s="49" t="n">
         <f aca="false">L20+L21+L22</f>
         <v>18500</v>
       </c>
-      <c r="M23" s="63" t="n">
+      <c r="M23" s="49" t="n">
         <f aca="false">M20+M21+M22</f>
         <v>18500</v>
       </c>
-      <c r="N23" s="63" t="n">
+      <c r="N23" s="49" t="n">
         <f aca="false">N20+N21+N22</f>
         <v>18500</v>
       </c>
-      <c r="O23" s="63" t="n">
+      <c r="O23" s="49" t="n">
         <f aca="false">O20+O21+O22</f>
         <v>21500</v>
       </c>
-      <c r="P23" s="63" t="n">
+      <c r="P23" s="49" t="n">
         <f aca="false">P20+P21+P22</f>
         <v>21500</v>
       </c>
-      <c r="Q23" s="63" t="n">
+      <c r="Q23" s="49" t="n">
         <f aca="false">Q20+Q21+Q22</f>
         <v>21500</v>
       </c>
-      <c r="R23" s="63" t="n">
+      <c r="R23" s="49" t="n">
         <f aca="false">R20+R21+R22</f>
         <v>21500</v>
       </c>
-      <c r="S23" s="63" t="n">
+      <c r="S23" s="49" t="n">
         <f aca="false">S20+S21+S22</f>
         <v>21500</v>
       </c>
-      <c r="T23" s="63" t="n">
+      <c r="T23" s="49" t="n">
         <f aca="false">T20+T21+T22</f>
         <v>21500</v>
       </c>
-      <c r="U23" s="63" t="n">
+      <c r="U23" s="49" t="n">
         <f aca="false">U20+U21+U22</f>
         <v>21500</v>
       </c>
-      <c r="V23" s="63" t="n">
+      <c r="V23" s="49" t="n">
         <f aca="false">V20+V21+V22</f>
         <v>21500</v>
       </c>
-      <c r="W23" s="63" t="n">
+      <c r="W23" s="49" t="n">
         <f aca="false">W20+W21+W22</f>
         <v>21500</v>
       </c>
-      <c r="X23" s="63" t="n">
+      <c r="X23" s="49" t="n">
         <f aca="false">X20+X21+X22</f>
         <v>21500</v>
       </c>
-      <c r="Y23" s="63" t="n">
+      <c r="Y23" s="49" t="n">
         <f aca="false">Y20+Y21+Y22</f>
         <v>21500</v>
       </c>
-      <c r="Z23" s="63" t="n">
+      <c r="Z23" s="49" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>300250</v>
-      </c>
-      <c r="AA23" s="63" t="n">
+        <v>281500</v>
+      </c>
+      <c r="AA23" s="49" t="n">
         <f aca="false">SUM(N23:Y23)</f>
         <v>255000</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>550</v>
       </c>
-      <c r="B25" s="50"/>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="50"/>
-      <c r="L25" s="50"/>
-      <c r="M25" s="50"/>
-      <c r="N25" s="50"/>
-      <c r="O25" s="50"/>
-      <c r="P25" s="50"/>
-      <c r="Q25" s="50"/>
-      <c r="R25" s="50"/>
-      <c r="S25" s="50"/>
-      <c r="T25" s="50"/>
-      <c r="U25" s="50"/>
-      <c r="V25" s="50"/>
-      <c r="W25" s="50"/>
-      <c r="X25" s="50"/>
-      <c r="Y25" s="50"/>
-      <c r="Z25" s="50"/>
-      <c r="AA25" s="50"/>
-      <c r="AB25" s="50"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="4"/>
+      <c r="V25" s="4"/>
+      <c r="W25" s="4"/>
+      <c r="X25" s="4"/>
+      <c r="Y25" s="4"/>
+      <c r="Z25" s="4"/>
+      <c r="AA25" s="4"/>
+      <c r="AB25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="B26" s="61" t="n">
+      <c r="B26" s="38" t="n">
         <f aca="false">IF(1&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="C26" s="61" t="n">
+      <c r="C26" s="38" t="n">
         <f aca="false">IF(2&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="D26" s="61" t="n">
+      <c r="D26" s="38" t="n">
         <f aca="false">IF(3&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="E26" s="61" t="n">
+      <c r="E26" s="38" t="n">
         <f aca="false">IF(4&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="F26" s="61" t="n">
+      <c r="F26" s="38" t="n">
         <f aca="false">IF(5&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="61" t="n">
+      <c r="G26" s="38" t="n">
         <f aca="false">IF(6&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="61" t="n">
+      <c r="H26" s="38" t="n">
         <f aca="false">IF(7&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="I26" s="61" t="n">
+      <c r="I26" s="38" t="n">
         <f aca="false">IF(8&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="61" t="n">
+      <c r="J26" s="38" t="n">
         <f aca="false">IF(9&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="61" t="n">
+      <c r="K26" s="38" t="n">
         <f aca="false">IF(10&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="L26" s="61" t="n">
+      <c r="L26" s="38" t="n">
         <f aca="false">IF(11&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="M26" s="61" t="n">
+      <c r="M26" s="38" t="n">
         <f aca="false">IF(12&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="N26" s="61" t="n">
+      <c r="N26" s="38" t="n">
         <f aca="false">IF(13&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="O26" s="61" t="n">
+      <c r="O26" s="38" t="n">
         <f aca="false">IF(14&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="P26" s="61" t="n">
+      <c r="P26" s="38" t="n">
         <f aca="false">IF(15&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Q26" s="61" t="n">
+      <c r="Q26" s="38" t="n">
         <f aca="false">IF(16&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="R26" s="61" t="n">
+      <c r="R26" s="38" t="n">
         <f aca="false">IF(17&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="S26" s="61" t="n">
+      <c r="S26" s="38" t="n">
         <f aca="false">IF(18&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="T26" s="61" t="n">
+      <c r="T26" s="38" t="n">
         <f aca="false">IF(19&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="U26" s="61" t="n">
+      <c r="U26" s="38" t="n">
         <f aca="false">IF(20&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="V26" s="61" t="n">
+      <c r="V26" s="38" t="n">
         <f aca="false">IF(21&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="W26" s="61" t="n">
+      <c r="W26" s="38" t="n">
         <f aca="false">IF(22&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="X26" s="61" t="n">
+      <c r="X26" s="38" t="n">
         <f aca="false">IF(23&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Y26" s="61" t="n">
+      <c r="Y26" s="38" t="n">
         <f aca="false">IF(24&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Z26" s="64" t="n">
+      <c r="Z26" s="18" t="n">
         <f aca="false">SUM(B26:M26)</f>
         <v>32000</v>
       </c>
-      <c r="AA26" s="64" t="n">
+      <c r="AA26" s="18" t="n">
         <f aca="false">SUM(N26:Y26)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B27" s="61" t="n">
+      <c r="B27" s="38" t="n">
         <f aca="false">IF(1=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="C27" s="61" t="n">
+      <c r="C27" s="38" t="n">
         <f aca="false">IF(2=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="D27" s="61" t="n">
+      <c r="D27" s="38" t="n">
         <f aca="false">IF(3=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="61" t="n">
+      <c r="E27" s="38" t="n">
         <f aca="false">IF(4=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="61" t="n">
+      <c r="F27" s="38" t="n">
         <f aca="false">IF(5=$B$5,$B$8,0)</f>
-        <v>106250</v>
-      </c>
-      <c r="G27" s="61" t="n">
+        <v>87500</v>
+      </c>
+      <c r="G27" s="38" t="n">
         <f aca="false">IF(6=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="H27" s="61" t="n">
+      <c r="H27" s="38" t="n">
         <f aca="false">IF(7=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="I27" s="61" t="n">
+      <c r="I27" s="38" t="n">
         <f aca="false">IF(8=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="J27" s="61" t="n">
+      <c r="J27" s="38" t="n">
         <f aca="false">IF(9=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="K27" s="61" t="n">
+      <c r="K27" s="38" t="n">
         <f aca="false">IF(10=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="L27" s="61" t="n">
+      <c r="L27" s="38" t="n">
         <f aca="false">IF(11=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="M27" s="61" t="n">
+      <c r="M27" s="38" t="n">
         <f aca="false">IF(12=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="N27" s="61" t="n">
+      <c r="N27" s="38" t="n">
         <f aca="false">IF(13=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="O27" s="61" t="n">
+      <c r="O27" s="38" t="n">
         <f aca="false">IF(14=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="P27" s="61" t="n">
+      <c r="P27" s="38" t="n">
         <f aca="false">IF(15=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Q27" s="61" t="n">
+      <c r="Q27" s="38" t="n">
         <f aca="false">IF(16=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="R27" s="61" t="n">
+      <c r="R27" s="38" t="n">
         <f aca="false">IF(17=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="S27" s="61" t="n">
+      <c r="S27" s="38" t="n">
         <f aca="false">IF(18=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="T27" s="61" t="n">
+      <c r="T27" s="38" t="n">
         <f aca="false">IF(19=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="U27" s="61" t="n">
+      <c r="U27" s="38" t="n">
         <f aca="false">IF(20=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="V27" s="61" t="n">
+      <c r="V27" s="38" t="n">
         <f aca="false">IF(21=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="W27" s="61" t="n">
+      <c r="W27" s="38" t="n">
         <f aca="false">IF(22=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="X27" s="61" t="n">
+      <c r="X27" s="38" t="n">
         <f aca="false">IF(23=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Y27" s="61" t="n">
+      <c r="Y27" s="38" t="n">
         <f aca="false">IF(24=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Z27" s="64" t="n">
+      <c r="Z27" s="18" t="n">
         <f aca="false">SUM(B27:M27)</f>
-        <v>106250</v>
-      </c>
-      <c r="AA27" s="64" t="n">
+        <v>87500</v>
+      </c>
+      <c r="AA27" s="18" t="n">
         <f aca="false">SUM(N27:Y27)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="B28" s="61" t="n">
+      <c r="B28" s="38" t="n">
         <f aca="false">IF(AND(1&gt;$B$5,1&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="C28" s="61" t="n">
+      <c r="C28" s="38" t="n">
         <f aca="false">IF(AND(2&gt;$B$5,2&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="D28" s="61" t="n">
+      <c r="D28" s="38" t="n">
         <f aca="false">IF(AND(3&gt;$B$5,3&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="61" t="n">
+      <c r="E28" s="38" t="n">
         <f aca="false">IF(AND(4&gt;$B$5,4&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="61" t="n">
+      <c r="F28" s="38" t="n">
         <f aca="false">IF(AND(5&gt;$B$5,5&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="61" t="n">
+      <c r="G28" s="38" t="n">
         <f aca="false">IF(AND(6&gt;$B$5,6&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="H28" s="61" t="n">
+      <c r="H28" s="38" t="n">
         <f aca="false">IF(AND(7&gt;$B$5,7&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="I28" s="61" t="n">
+      <c r="I28" s="38" t="n">
         <f aca="false">IF(AND(8&gt;$B$5,8&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="J28" s="61" t="n">
+      <c r="J28" s="38" t="n">
         <f aca="false">IF(AND(9&gt;$B$5,9&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="K28" s="61" t="n">
+      <c r="K28" s="38" t="n">
         <f aca="false">IF(AND(10&gt;$B$5,10&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="L28" s="61" t="n">
+      <c r="L28" s="38" t="n">
         <f aca="false">IF(AND(11&gt;$B$5,11&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="M28" s="61" t="n">
+      <c r="M28" s="38" t="n">
         <f aca="false">IF(AND(12&gt;$B$5,12&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="N28" s="61" t="n">
+      <c r="N28" s="38" t="n">
         <f aca="false">IF(AND(13&gt;$B$5,13&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="O28" s="61" t="n">
+      <c r="O28" s="38" t="n">
         <f aca="false">IF(AND(14&gt;$B$5,14&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="P28" s="61" t="n">
+      <c r="P28" s="38" t="n">
         <f aca="false">IF(AND(15&gt;$B$5,15&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="Q28" s="61" t="n">
+      <c r="Q28" s="38" t="n">
         <f aca="false">IF(AND(16&gt;$B$5,16&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="R28" s="61" t="n">
+      <c r="R28" s="38" t="n">
         <f aca="false">IF(AND(17&gt;$B$5,17&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="S28" s="61" t="n">
+      <c r="S28" s="38" t="n">
         <f aca="false">IF(AND(18&gt;$B$5,18&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="T28" s="61" t="n">
+      <c r="T28" s="38" t="n">
         <f aca="false">IF(AND(19&gt;$B$5,19&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="U28" s="61" t="n">
+      <c r="U28" s="38" t="n">
         <f aca="false">IF(AND(20&gt;$B$5,20&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="V28" s="61" t="n">
+      <c r="V28" s="38" t="n">
         <f aca="false">IF(AND(21&gt;$B$5,21&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="W28" s="61" t="n">
+      <c r="W28" s="38" t="n">
         <f aca="false">IF(AND(22&gt;$B$5,22&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="X28" s="61" t="n">
+      <c r="X28" s="38" t="n">
         <f aca="false">IF(AND(23&gt;$B$5,23&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>6000</v>
       </c>
-      <c r="Y28" s="61" t="n">
+      <c r="Y28" s="38" t="n">
         <f aca="false">IF(AND(24&gt;$B$5,24&lt;=$B$5+$B$10),$B$9,0)</f>
         <v>0</v>
       </c>
-      <c r="Z28" s="64" t="n">
+      <c r="Z28" s="18" t="n">
         <f aca="false">SUM(B28:M28)</f>
         <v>42000</v>
       </c>
-      <c r="AA28" s="64" t="n">
+      <c r="AA28" s="18" t="n">
         <f aca="false">SUM(N28:Y28)</f>
         <v>66000</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="B29" s="61" t="n">
+      <c r="B29" s="38" t="n">
         <v>3500</v>
       </c>
-      <c r="C29" s="61" t="n">
+      <c r="C29" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="D29" s="61" t="n">
+      <c r="D29" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="E29" s="61" t="n">
+      <c r="E29" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="F29" s="61" t="n">
+      <c r="F29" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="G29" s="61" t="n">
+      <c r="G29" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="H29" s="61" t="n">
+      <c r="H29" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="I29" s="61" t="n">
+      <c r="I29" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="J29" s="61" t="n">
+      <c r="J29" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="K29" s="61" t="n">
+      <c r="K29" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="L29" s="61" t="n">
+      <c r="L29" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="M29" s="61" t="n">
+      <c r="M29" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="N29" s="61" t="n">
+      <c r="N29" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="O29" s="61" t="n">
+      <c r="O29" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="P29" s="61" t="n">
+      <c r="P29" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="Q29" s="61" t="n">
+      <c r="Q29" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="R29" s="61" t="n">
+      <c r="R29" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="S29" s="61" t="n">
+      <c r="S29" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="T29" s="61" t="n">
+      <c r="T29" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="U29" s="61" t="n">
+      <c r="U29" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="V29" s="61" t="n">
+      <c r="V29" s="38" t="n">
         <v>17000</v>
       </c>
-      <c r="W29" s="61" t="n">
+      <c r="W29" s="38" t="n">
         <v>17000</v>
       </c>
-      <c r="X29" s="61" t="n">
+      <c r="X29" s="38" t="n">
         <v>14000</v>
       </c>
-      <c r="Y29" s="61" t="n">
+      <c r="Y29" s="38" t="n">
         <v>14000</v>
       </c>
-      <c r="Z29" s="64" t="n">
+      <c r="Z29" s="18" t="n">
         <f aca="false">SUM(B29:M29)</f>
         <v>104000</v>
       </c>
-      <c r="AA29" s="64" t="n">
+      <c r="AA29" s="18" t="n">
         <f aca="false">SUM(N29:Y29)</f>
         <v>188500</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="B30" s="64" t="n">
+      <c r="B30" s="18" t="n">
         <f aca="false">IF(1&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="C30" s="64" t="n">
+      <c r="C30" s="18" t="n">
         <f aca="false">IF(2&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="D30" s="64" t="n">
+      <c r="D30" s="18" t="n">
         <f aca="false">IF(3&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="64" t="n">
+      <c r="E30" s="18" t="n">
         <f aca="false">IF(4&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="64" t="n">
+      <c r="F30" s="18" t="n">
         <f aca="false">IF(5&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="G30" s="64" t="n">
+      <c r="G30" s="18" t="n">
         <f aca="false">IF(6&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="H30" s="64" t="n">
+      <c r="H30" s="18" t="n">
         <f aca="false">IF(7&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="I30" s="64" t="n">
+      <c r="I30" s="18" t="n">
         <f aca="false">IF(8&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="J30" s="64" t="n">
+      <c r="J30" s="18" t="n">
         <f aca="false">IF(9&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="K30" s="64" t="n">
+      <c r="K30" s="18" t="n">
         <f aca="false">IF(10&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="L30" s="64" t="n">
+      <c r="L30" s="18" t="n">
         <f aca="false">IF(11&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="M30" s="64" t="n">
+      <c r="M30" s="18" t="n">
         <f aca="false">IF(12&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="N30" s="64" t="n">
+      <c r="N30" s="18" t="n">
         <f aca="false">IF(13&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="O30" s="64" t="n">
+      <c r="O30" s="18" t="n">
         <f aca="false">IF(14&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="P30" s="64" t="n">
+      <c r="P30" s="18" t="n">
         <f aca="false">IF(15&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Q30" s="64" t="n">
+      <c r="Q30" s="18" t="n">
         <f aca="false">IF(16&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="R30" s="64" t="n">
+      <c r="R30" s="18" t="n">
         <f aca="false">IF(17&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="S30" s="64" t="n">
+      <c r="S30" s="18" t="n">
         <f aca="false">IF(18&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="T30" s="64" t="n">
+      <c r="T30" s="18" t="n">
         <f aca="false">IF(19&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="U30" s="64" t="n">
+      <c r="U30" s="18" t="n">
         <f aca="false">IF(20&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="V30" s="64" t="n">
+      <c r="V30" s="18" t="n">
         <f aca="false">IF(21&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="W30" s="64" t="n">
+      <c r="W30" s="18" t="n">
         <f aca="false">IF(22&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="X30" s="64" t="n">
+      <c r="X30" s="18" t="n">
         <f aca="false">IF(23&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Y30" s="64" t="n">
+      <c r="Y30" s="18" t="n">
         <f aca="false">IF(24&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Z30" s="64" t="n">
+      <c r="Z30" s="18" t="n">
         <f aca="false">SUM(B30:M30)</f>
         <v>-19200</v>
       </c>
-      <c r="AA30" s="64" t="n">
+      <c r="AA30" s="18" t="n">
         <f aca="false">SUM(N30:Y30)</f>
         <v>-28800</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="62" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24" t="s">
         <v>555</v>
       </c>
-      <c r="B31" s="65" t="n">
+      <c r="B31" s="19" t="n">
         <f aca="false">B26+B27+B28+B29+B30</f>
         <v>11500</v>
       </c>
-      <c r="C31" s="65" t="n">
+      <c r="C31" s="19" t="n">
         <f aca="false">C26+C27+C28+C29+C30</f>
         <v>13000</v>
       </c>
-      <c r="D31" s="65" t="n">
+      <c r="D31" s="19" t="n">
         <f aca="false">D26+D27+D28+D29+D30</f>
         <v>13000</v>
       </c>
-      <c r="E31" s="65" t="n">
+      <c r="E31" s="19" t="n">
         <f aca="false">E26+E27+E28+E29+E30</f>
         <v>16000</v>
       </c>
-      <c r="F31" s="65" t="n">
+      <c r="F31" s="19" t="n">
         <f aca="false">F26+F27+F28+F29+F30</f>
-        <v>111850</v>
-      </c>
-      <c r="G31" s="65" t="n">
+        <v>93100</v>
+      </c>
+      <c r="G31" s="19" t="n">
         <f aca="false">G26+G27+G28+G29+G30</f>
         <v>11600</v>
       </c>
-      <c r="H31" s="65" t="n">
+      <c r="H31" s="19" t="n">
         <f aca="false">H26+H27+H28+H29+H30</f>
         <v>11600</v>
       </c>
-      <c r="I31" s="65" t="n">
+      <c r="I31" s="19" t="n">
         <f aca="false">I26+I27+I28+I29+I30</f>
         <v>14100</v>
       </c>
-      <c r="J31" s="65" t="n">
+      <c r="J31" s="19" t="n">
         <f aca="false">J26+J27+J28+J29+J30</f>
         <v>14100</v>
       </c>
-      <c r="K31" s="65" t="n">
+      <c r="K31" s="19" t="n">
         <f aca="false">K26+K27+K28+K29+K30</f>
         <v>14100</v>
       </c>
-      <c r="L31" s="65" t="n">
+      <c r="L31" s="19" t="n">
         <f aca="false">L26+L27+L28+L29+L30</f>
         <v>17100</v>
       </c>
-      <c r="M31" s="65" t="n">
+      <c r="M31" s="19" t="n">
         <f aca="false">M26+M27+M28+M29+M30</f>
         <v>17100</v>
       </c>
-      <c r="N31" s="65" t="n">
+      <c r="N31" s="19" t="n">
         <f aca="false">N26+N27+N28+N29+N30</f>
         <v>17100</v>
       </c>
-      <c r="O31" s="65" t="n">
+      <c r="O31" s="19" t="n">
         <f aca="false">O26+O27+O28+O29+O30</f>
         <v>17100</v>
       </c>
-      <c r="P31" s="65" t="n">
+      <c r="P31" s="19" t="n">
         <f aca="false">P26+P27+P28+P29+P30</f>
         <v>17100</v>
       </c>
-      <c r="Q31" s="65" t="n">
+      <c r="Q31" s="19" t="n">
         <f aca="false">Q26+Q27+Q28+Q29+Q30</f>
         <v>20100</v>
       </c>
-      <c r="R31" s="65" t="n">
+      <c r="R31" s="19" t="n">
         <f aca="false">R26+R27+R28+R29+R30</f>
         <v>20100</v>
       </c>
-      <c r="S31" s="65" t="n">
+      <c r="S31" s="19" t="n">
         <f aca="false">S26+S27+S28+S29+S30</f>
         <v>20100</v>
       </c>
-      <c r="T31" s="65" t="n">
+      <c r="T31" s="19" t="n">
         <f aca="false">T26+T27+T28+T29+T30</f>
         <v>20100</v>
       </c>
-      <c r="U31" s="65" t="n">
+      <c r="U31" s="19" t="n">
         <f aca="false">U26+U27+U28+U29+U30</f>
         <v>23600</v>
       </c>
-      <c r="V31" s="65" t="n">
+      <c r="V31" s="19" t="n">
         <f aca="false">V26+V27+V28+V29+V30</f>
         <v>20600</v>
       </c>
-      <c r="W31" s="65" t="n">
+      <c r="W31" s="19" t="n">
         <f aca="false">W26+W27+W28+W29+W30</f>
         <v>20600</v>
       </c>
-      <c r="X31" s="65" t="n">
+      <c r="X31" s="19" t="n">
         <f aca="false">X26+X27+X28+X29+X30</f>
         <v>17600</v>
       </c>
-      <c r="Y31" s="65" t="n">
+      <c r="Y31" s="19" t="n">
         <f aca="false">Y26+Y27+Y28+Y29+Y30</f>
         <v>11600</v>
       </c>
-      <c r="Z31" s="65" t="n">
+      <c r="Z31" s="19" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>265050</v>
-      </c>
-      <c r="AA31" s="65" t="n">
+        <v>246300</v>
+      </c>
+      <c r="AA31" s="19" t="n">
         <f aca="false">SUM(N31:Y31)</f>
         <v>225700</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="50" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>556</v>
       </c>
-      <c r="B33" s="50"/>
-      <c r="C33" s="50"/>
-      <c r="D33" s="50"/>
-      <c r="E33" s="50"/>
-      <c r="F33" s="50"/>
-      <c r="G33" s="50"/>
-      <c r="H33" s="50"/>
-      <c r="I33" s="50"/>
-      <c r="J33" s="50"/>
-      <c r="K33" s="50"/>
-      <c r="L33" s="50"/>
-      <c r="M33" s="50"/>
-      <c r="N33" s="50"/>
-      <c r="O33" s="50"/>
-      <c r="P33" s="50"/>
-      <c r="Q33" s="50"/>
-      <c r="R33" s="50"/>
-      <c r="S33" s="50"/>
-      <c r="T33" s="50"/>
-      <c r="U33" s="50"/>
-      <c r="V33" s="50"/>
-      <c r="W33" s="50"/>
-      <c r="X33" s="50"/>
-      <c r="Y33" s="50"/>
-      <c r="Z33" s="50"/>
-      <c r="AA33" s="50"/>
-      <c r="AB33" s="50"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
+      <c r="S33" s="4"/>
+      <c r="T33" s="4"/>
+      <c r="U33" s="4"/>
+      <c r="V33" s="4"/>
+      <c r="W33" s="4"/>
+      <c r="X33" s="4"/>
+      <c r="Y33" s="4"/>
+      <c r="Z33" s="4"/>
+      <c r="AA33" s="4"/>
+      <c r="AB33" s="4"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="B34" s="61" t="n">
+      <c r="B34" s="38" t="n">
         <f aca="false">IF(1&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="C34" s="61" t="n">
+      <c r="C34" s="38" t="n">
         <f aca="false">IF(2&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="D34" s="61" t="n">
+      <c r="D34" s="38" t="n">
         <f aca="false">IF(3&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="E34" s="61" t="n">
+      <c r="E34" s="38" t="n">
         <f aca="false">IF(4&lt;$B$5,8000,0)</f>
         <v>8000</v>
       </c>
-      <c r="F34" s="61" t="n">
+      <c r="F34" s="38" t="n">
         <f aca="false">IF(5&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="G34" s="61" t="n">
+      <c r="G34" s="38" t="n">
         <f aca="false">IF(6&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="H34" s="61" t="n">
+      <c r="H34" s="38" t="n">
         <f aca="false">IF(7&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="I34" s="61" t="n">
+      <c r="I34" s="38" t="n">
         <f aca="false">IF(8&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="J34" s="61" t="n">
+      <c r="J34" s="38" t="n">
         <f aca="false">IF(9&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="K34" s="61" t="n">
+      <c r="K34" s="38" t="n">
         <f aca="false">IF(10&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="L34" s="61" t="n">
+      <c r="L34" s="38" t="n">
         <f aca="false">IF(11&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="M34" s="61" t="n">
+      <c r="M34" s="38" t="n">
         <f aca="false">IF(12&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="N34" s="61" t="n">
+      <c r="N34" s="38" t="n">
         <f aca="false">IF(13&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="O34" s="61" t="n">
+      <c r="O34" s="38" t="n">
         <f aca="false">IF(14&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="P34" s="61" t="n">
+      <c r="P34" s="38" t="n">
         <f aca="false">IF(15&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Q34" s="61" t="n">
+      <c r="Q34" s="38" t="n">
         <f aca="false">IF(16&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="R34" s="61" t="n">
+      <c r="R34" s="38" t="n">
         <f aca="false">IF(17&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="S34" s="61" t="n">
+      <c r="S34" s="38" t="n">
         <f aca="false">IF(18&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="T34" s="61" t="n">
+      <c r="T34" s="38" t="n">
         <f aca="false">IF(19&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="U34" s="61" t="n">
+      <c r="U34" s="38" t="n">
         <f aca="false">IF(20&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="V34" s="61" t="n">
+      <c r="V34" s="38" t="n">
         <f aca="false">IF(21&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="W34" s="61" t="n">
+      <c r="W34" s="38" t="n">
         <f aca="false">IF(22&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="X34" s="61" t="n">
+      <c r="X34" s="38" t="n">
         <f aca="false">IF(23&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Y34" s="61" t="n">
+      <c r="Y34" s="38" t="n">
         <f aca="false">IF(24&lt;$B$5,8000,0)</f>
         <v>0</v>
       </c>
-      <c r="Z34" s="64" t="n">
+      <c r="Z34" s="18" t="n">
         <f aca="false">SUM(B34:M34)</f>
         <v>32000</v>
       </c>
-      <c r="AA34" s="64" t="n">
+      <c r="AA34" s="18" t="n">
         <f aca="false">SUM(N34:Y34)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B35" s="61" t="n">
+      <c r="B35" s="38" t="n">
         <f aca="false">IF(1=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="C35" s="61" t="n">
+      <c r="C35" s="38" t="n">
         <f aca="false">IF(2=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="D35" s="61" t="n">
+      <c r="D35" s="38" t="n">
         <f aca="false">IF(3=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="61" t="n">
+      <c r="E35" s="38" t="n">
         <f aca="false">IF(4=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="F35" s="61" t="n">
+      <c r="F35" s="38" t="n">
         <f aca="false">IF(5=$B$5,$B$8,0)</f>
-        <v>106250</v>
-      </c>
-      <c r="G35" s="61" t="n">
+        <v>87500</v>
+      </c>
+      <c r="G35" s="38" t="n">
         <f aca="false">IF(6=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="61" t="n">
+      <c r="H35" s="38" t="n">
         <f aca="false">IF(7=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="I35" s="61" t="n">
+      <c r="I35" s="38" t="n">
         <f aca="false">IF(8=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="J35" s="61" t="n">
+      <c r="J35" s="38" t="n">
         <f aca="false">IF(9=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="K35" s="61" t="n">
+      <c r="K35" s="38" t="n">
         <f aca="false">IF(10=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="L35" s="61" t="n">
+      <c r="L35" s="38" t="n">
         <f aca="false">IF(11=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="M35" s="61" t="n">
+      <c r="M35" s="38" t="n">
         <f aca="false">IF(12=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="N35" s="61" t="n">
+      <c r="N35" s="38" t="n">
         <f aca="false">IF(13=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="O35" s="61" t="n">
+      <c r="O35" s="38" t="n">
         <f aca="false">IF(14=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="P35" s="61" t="n">
+      <c r="P35" s="38" t="n">
         <f aca="false">IF(15=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Q35" s="61" t="n">
+      <c r="Q35" s="38" t="n">
         <f aca="false">IF(16=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="R35" s="61" t="n">
+      <c r="R35" s="38" t="n">
         <f aca="false">IF(17=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="S35" s="61" t="n">
+      <c r="S35" s="38" t="n">
         <f aca="false">IF(18=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="T35" s="61" t="n">
+      <c r="T35" s="38" t="n">
         <f aca="false">IF(19=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="U35" s="61" t="n">
+      <c r="U35" s="38" t="n">
         <f aca="false">IF(20=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="V35" s="61" t="n">
+      <c r="V35" s="38" t="n">
         <f aca="false">IF(21=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="W35" s="61" t="n">
+      <c r="W35" s="38" t="n">
         <f aca="false">IF(22=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="X35" s="61" t="n">
+      <c r="X35" s="38" t="n">
         <f aca="false">IF(23=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Y35" s="61" t="n">
+      <c r="Y35" s="38" t="n">
         <f aca="false">IF(24=$B$5,$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="Z35" s="64" t="n">
+      <c r="Z35" s="18" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>106250</v>
-      </c>
-      <c r="AA35" s="64" t="n">
+        <v>87500</v>
+      </c>
+      <c r="AA35" s="18" t="n">
         <f aca="false">SUM(N35:Y35)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="B36" s="61" t="n">
+      <c r="B36" s="38" t="n">
         <v>3500</v>
       </c>
-      <c r="C36" s="61" t="n">
+      <c r="C36" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="D36" s="61" t="n">
+      <c r="D36" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="E36" s="61" t="n">
+      <c r="E36" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="F36" s="61" t="n">
+      <c r="F36" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="G36" s="61" t="n">
+      <c r="G36" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="H36" s="61" t="n">
+      <c r="H36" s="38" t="n">
         <v>8000</v>
       </c>
-      <c r="I36" s="61" t="n">
+      <c r="I36" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="J36" s="61" t="n">
+      <c r="J36" s="38" t="n">
         <v>10500</v>
       </c>
-      <c r="K36" s="61" t="n">
+      <c r="K36" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="L36" s="61" t="n">
+      <c r="L36" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="M36" s="61" t="n">
+      <c r="M36" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="N36" s="61" t="n">
+      <c r="N36" s="38" t="n">
         <v>13500</v>
       </c>
-      <c r="O36" s="61" t="n">
+      <c r="O36" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="P36" s="61" t="n">
+      <c r="P36" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="Q36" s="61" t="n">
+      <c r="Q36" s="38" t="n">
         <v>16500</v>
       </c>
-      <c r="R36" s="61" t="n">
+      <c r="R36" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="S36" s="61" t="n">
+      <c r="S36" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="T36" s="61" t="n">
+      <c r="T36" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="U36" s="61" t="n">
+      <c r="U36" s="38" t="n">
         <v>23000</v>
       </c>
-      <c r="V36" s="61" t="n">
+      <c r="V36" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="W36" s="61" t="n">
+      <c r="W36" s="38" t="n">
         <v>20000</v>
       </c>
-      <c r="X36" s="61" t="n">
+      <c r="X36" s="38" t="n">
         <v>20500</v>
       </c>
-      <c r="Y36" s="61" t="n">
+      <c r="Y36" s="38" t="n">
         <v>20500</v>
       </c>
-      <c r="Z36" s="64" t="n">
+      <c r="Z36" s="18" t="n">
         <f aca="false">SUM(B36:M36)</f>
         <v>107000</v>
       </c>
-      <c r="AA36" s="64" t="n">
+      <c r="AA36" s="18" t="n">
         <f aca="false">SUM(N36:Y36)</f>
         <v>227000</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="B37" s="64" t="n">
+      <c r="B37" s="18" t="n">
         <f aca="false">IF(1&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="C37" s="64" t="n">
+      <c r="C37" s="18" t="n">
         <f aca="false">IF(2&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="D37" s="64" t="n">
+      <c r="D37" s="18" t="n">
         <f aca="false">IF(3&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="E37" s="64" t="n">
+      <c r="E37" s="18" t="n">
         <f aca="false">IF(4&gt;=$B$11,-$B$12,0)</f>
         <v>0</v>
       </c>
-      <c r="F37" s="64" t="n">
+      <c r="F37" s="18" t="n">
         <f aca="false">IF(5&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="G37" s="64" t="n">
+      <c r="G37" s="18" t="n">
         <f aca="false">IF(6&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="H37" s="64" t="n">
+      <c r="H37" s="18" t="n">
         <f aca="false">IF(7&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="I37" s="64" t="n">
+      <c r="I37" s="18" t="n">
         <f aca="false">IF(8&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="J37" s="64" t="n">
+      <c r="J37" s="18" t="n">
         <f aca="false">IF(9&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="K37" s="64" t="n">
+      <c r="K37" s="18" t="n">
         <f aca="false">IF(10&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="L37" s="64" t="n">
+      <c r="L37" s="18" t="n">
         <f aca="false">IF(11&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="M37" s="64" t="n">
+      <c r="M37" s="18" t="n">
         <f aca="false">IF(12&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="N37" s="64" t="n">
+      <c r="N37" s="18" t="n">
         <f aca="false">IF(13&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="O37" s="64" t="n">
+      <c r="O37" s="18" t="n">
         <f aca="false">IF(14&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="P37" s="64" t="n">
+      <c r="P37" s="18" t="n">
         <f aca="false">IF(15&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Q37" s="64" t="n">
+      <c r="Q37" s="18" t="n">
         <f aca="false">IF(16&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="R37" s="64" t="n">
+      <c r="R37" s="18" t="n">
         <f aca="false">IF(17&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="S37" s="64" t="n">
+      <c r="S37" s="18" t="n">
         <f aca="false">IF(18&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="T37" s="64" t="n">
+      <c r="T37" s="18" t="n">
         <f aca="false">IF(19&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="U37" s="64" t="n">
+      <c r="U37" s="18" t="n">
         <f aca="false">IF(20&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="V37" s="64" t="n">
+      <c r="V37" s="18" t="n">
         <f aca="false">IF(21&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="W37" s="64" t="n">
+      <c r="W37" s="18" t="n">
         <f aca="false">IF(22&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="X37" s="64" t="n">
+      <c r="X37" s="18" t="n">
         <f aca="false">IF(23&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Y37" s="64" t="n">
+      <c r="Y37" s="18" t="n">
         <f aca="false">IF(24&gt;=$B$11,-$B$12,0)</f>
         <v>-2400</v>
       </c>
-      <c r="Z37" s="64" t="n">
+      <c r="Z37" s="18" t="n">
         <f aca="false">SUM(B37:M37)</f>
         <v>-19200</v>
       </c>
-      <c r="AA37" s="64" t="n">
+      <c r="AA37" s="18" t="n">
         <f aca="false">SUM(N37:Y37)</f>
         <v>-28800</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="62" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="24" t="s">
         <v>559</v>
       </c>
-      <c r="B38" s="65" t="n">
+      <c r="B38" s="19" t="n">
         <f aca="false">B34+B35+B36+B37</f>
         <v>11500</v>
       </c>
-      <c r="C38" s="65" t="n">
+      <c r="C38" s="19" t="n">
         <f aca="false">C34+C35+C36+C37</f>
         <v>13000</v>
       </c>
-      <c r="D38" s="65" t="n">
+      <c r="D38" s="19" t="n">
         <f aca="false">D34+D35+D36+D37</f>
         <v>13000</v>
       </c>
-      <c r="E38" s="65" t="n">
+      <c r="E38" s="19" t="n">
         <f aca="false">E34+E35+E36+E37</f>
         <v>16000</v>
       </c>
-      <c r="F38" s="65" t="n">
+      <c r="F38" s="19" t="n">
         <f aca="false">F34+F35+F36+F37</f>
-        <v>111850</v>
-      </c>
-      <c r="G38" s="65" t="n">
+        <v>93100</v>
+      </c>
+      <c r="G38" s="19" t="n">
         <f aca="false">G34+G35+G36+G37</f>
         <v>5600</v>
       </c>
-      <c r="H38" s="65" t="n">
+      <c r="H38" s="19" t="n">
         <f aca="false">H34+H35+H36+H37</f>
         <v>5600</v>
       </c>
-      <c r="I38" s="65" t="n">
+      <c r="I38" s="19" t="n">
         <f aca="false">I34+I35+I36+I37</f>
         <v>8100</v>
       </c>
-      <c r="J38" s="65" t="n">
+      <c r="J38" s="19" t="n">
         <f aca="false">J34+J35+J36+J37</f>
         <v>8100</v>
       </c>
-      <c r="K38" s="65" t="n">
+      <c r="K38" s="19" t="n">
         <f aca="false">K34+K35+K36+K37</f>
         <v>11100</v>
       </c>
-      <c r="L38" s="65" t="n">
+      <c r="L38" s="19" t="n">
         <f aca="false">L34+L35+L36+L37</f>
         <v>11100</v>
       </c>
-      <c r="M38" s="65" t="n">
+      <c r="M38" s="19" t="n">
         <f aca="false">M34+M35+M36+M37</f>
         <v>11100</v>
       </c>
-      <c r="N38" s="65" t="n">
+      <c r="N38" s="19" t="n">
         <f aca="false">N34+N35+N36+N37</f>
         <v>11100</v>
       </c>
-      <c r="O38" s="65" t="n">
+      <c r="O38" s="19" t="n">
         <f aca="false">O34+O35+O36+O37</f>
         <v>14100</v>
       </c>
-      <c r="P38" s="65" t="n">
+      <c r="P38" s="19" t="n">
         <f aca="false">P34+P35+P36+P37</f>
         <v>14100</v>
       </c>
-      <c r="Q38" s="65" t="n">
+      <c r="Q38" s="19" t="n">
         <f aca="false">Q34+Q35+Q36+Q37</f>
         <v>14100</v>
       </c>
-      <c r="R38" s="65" t="n">
+      <c r="R38" s="19" t="n">
         <f aca="false">R34+R35+R36+R37</f>
         <v>17600</v>
       </c>
-      <c r="S38" s="65" t="n">
+      <c r="S38" s="19" t="n">
         <f aca="false">S34+S35+S36+S37</f>
         <v>17600</v>
       </c>
-      <c r="T38" s="65" t="n">
+      <c r="T38" s="19" t="n">
         <f aca="false">T34+T35+T36+T37</f>
         <v>17600</v>
       </c>
-      <c r="U38" s="65" t="n">
+      <c r="U38" s="19" t="n">
         <f aca="false">U34+U35+U36+U37</f>
         <v>20600</v>
       </c>
-      <c r="V38" s="65" t="n">
+      <c r="V38" s="19" t="n">
         <f aca="false">V34+V35+V36+V37</f>
         <v>17600</v>
       </c>
-      <c r="W38" s="65" t="n">
+      <c r="W38" s="19" t="n">
         <f aca="false">W34+W35+W36+W37</f>
         <v>17600</v>
       </c>
-      <c r="X38" s="65" t="n">
+      <c r="X38" s="19" t="n">
         <f aca="false">X34+X35+X36+X37</f>
         <v>18100</v>
       </c>
-      <c r="Y38" s="65" t="n">
+      <c r="Y38" s="19" t="n">
         <f aca="false">Y34+Y35+Y36+Y37</f>
         <v>18100</v>
       </c>
-      <c r="Z38" s="65" t="n">
+      <c r="Z38" s="19" t="n">
         <f aca="false">SUM(B38:M38)</f>
-        <v>226050</v>
-      </c>
-      <c r="AA38" s="65" t="n">
+        <v>207300</v>
+      </c>
+      <c r="AA38" s="19" t="n">
         <f aca="false">SUM(N38:Y38)</f>
         <v>198200</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="50" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
         <v>560</v>
       </c>
-      <c r="B40" s="50"/>
-      <c r="C40" s="50"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="50"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="30" t="s">
         <v>132</v>
       </c>
@@ -6540,175 +6512,175 @@
         <v>401</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="B42" s="66" t="n">
+      <c r="B42" s="50" t="n">
         <f aca="false">Z23</f>
-        <v>300250</v>
-      </c>
-      <c r="C42" s="66" t="n">
+        <v>281500</v>
+      </c>
+      <c r="C42" s="50" t="n">
         <f aca="false">AA23</f>
         <v>255000</v>
       </c>
-      <c r="D42" s="66" t="n">
+      <c r="D42" s="50" t="n">
         <f aca="false">B42+C42</f>
-        <v>555250</v>
-      </c>
-      <c r="E42" s="0" t="s">
+        <v>536500</v>
+      </c>
+      <c r="E42" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="F42" s="0" t="s">
+      <c r="F42" s="1" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="67" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="51" t="s">
         <v>568</v>
       </c>
-      <c r="B43" s="68" t="n">
+      <c r="B43" s="52" t="n">
         <f aca="false">Z31</f>
-        <v>265050</v>
-      </c>
-      <c r="C43" s="68" t="n">
+        <v>246300</v>
+      </c>
+      <c r="C43" s="52" t="n">
         <f aca="false">AA31</f>
         <v>225700</v>
       </c>
-      <c r="D43" s="68" t="n">
+      <c r="D43" s="52" t="n">
         <f aca="false">B43+C43</f>
-        <v>490750</v>
-      </c>
-      <c r="E43" s="67" t="s">
+        <v>472000</v>
+      </c>
+      <c r="E43" s="51" t="s">
         <v>569</v>
       </c>
-      <c r="F43" s="67" t="s">
+      <c r="F43" s="51" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
         <v>571</v>
       </c>
-      <c r="B44" s="66" t="n">
+      <c r="B44" s="50" t="n">
         <f aca="false">Z38</f>
-        <v>226050</v>
-      </c>
-      <c r="C44" s="66" t="n">
+        <v>207300</v>
+      </c>
+      <c r="C44" s="50" t="n">
         <f aca="false">AA38</f>
         <v>198200</v>
       </c>
-      <c r="D44" s="66" t="n">
+      <c r="D44" s="50" t="n">
         <f aca="false">B44+C44</f>
-        <v>424250</v>
-      </c>
-      <c r="E44" s="0" t="s">
+        <v>405500</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="F44" s="0" t="s">
+      <c r="F44" s="1" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="50" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="B46" s="50"/>
-      <c r="C46" s="50"/>
-      <c r="D46" s="50"/>
-      <c r="E46" s="50"/>
-      <c r="F46" s="50"/>
-      <c r="G46" s="50"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="B47" s="69" t="n">
+      <c r="B47" s="41" t="n">
         <f aca="false">B15</f>
         <v>21</v>
       </c>
-      <c r="C47" s="52" t="s">
+      <c r="C47" s="6" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B48" s="69" t="n">
+      <c r="B48" s="41" t="n">
         <f aca="false">3*18</f>
         <v>54</v>
       </c>
-      <c r="C48" s="52" t="s">
+      <c r="C48" s="6" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B49" s="69" t="n">
+      <c r="B49" s="41" t="n">
         <f aca="false">173/12</f>
         <v>14.4166666666667</v>
       </c>
-      <c r="C49" s="52" t="s">
+      <c r="C49" s="6" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="s">
         <v>581</v>
       </c>
-      <c r="B50" s="69" t="n">
+      <c r="B50" s="41" t="n">
         <v>30</v>
       </c>
-      <c r="C50" s="52" t="s">
+      <c r="C50" s="6" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="62" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="24" t="s">
         <v>583</v>
       </c>
-      <c r="B51" s="70" t="n">
+      <c r="B51" s="53" t="n">
         <f aca="false">B47+B48+B49+B50</f>
         <v>119.416666666667</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="B52" s="69" t="n">
+      <c r="B52" s="41" t="n">
         <v>180</v>
       </c>
-      <c r="C52" s="52" t="s">
+      <c r="C52" s="6" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="62" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="24" t="s">
         <v>586</v>
       </c>
-      <c r="B53" s="71" t="n">
+      <c r="B53" s="54" t="n">
         <f aca="false">B52-B51</f>
         <v>60.5833333333333</v>
       </c>
-      <c r="C53" s="52" t="s">
+      <c r="C53" s="6" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="50" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
         <v>588</v>
       </c>
-      <c r="B55" s="50"/>
-      <c r="C55" s="50"/>
-      <c r="D55" s="50"/>
-      <c r="E55" s="50"/>
-      <c r="F55" s="50"/>
-      <c r="G55" s="50"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="27" t="s">
@@ -6881,8 +6853,89 @@
       <c r="N64" s="27"/>
       <c r="O64" s="27"/>
     </row>
+    <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="27" t="s">
+        <v>598</v>
+      </c>
+      <c r="B65" s="27"/>
+      <c r="C65" s="27"/>
+      <c r="D65" s="27"/>
+      <c r="E65" s="27"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="27"/>
+      <c r="H65" s="27"/>
+      <c r="I65" s="27"/>
+      <c r="J65" s="27"/>
+      <c r="K65" s="27"/>
+      <c r="L65" s="27"/>
+      <c r="M65" s="27"/>
+      <c r="N65" s="27"/>
+      <c r="O65" s="27"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="55" t="s">
+        <v>599</v>
+      </c>
+      <c r="B76" s="55"/>
+      <c r="C76" s="55"/>
+      <c r="D76" s="55"/>
+      <c r="E76" s="55"/>
+      <c r="F76" s="55"/>
+      <c r="G76" s="55"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="B77" s="56" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="B78" s="56" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="B79" s="56" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="57" t="s">
+        <v>603</v>
+      </c>
+      <c r="B80" s="58" t="n">
+        <f aca="false">B42*B77+B43*B78+B44*B79</f>
+        <v>241450</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="57" t="s">
+        <v>604</v>
+      </c>
+      <c r="B81" s="58" t="n">
+        <f aca="false">C42*B77+C43*B78+C44*B79</f>
+        <v>223400</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="57" t="s">
+        <v>605</v>
+      </c>
+      <c r="B82" s="58" t="n">
+        <f aca="false">B80+B81</f>
+        <v>464850</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="20">
     <mergeCell ref="A1:AA1"/>
     <mergeCell ref="A2:AA2"/>
     <mergeCell ref="A4:F4"/>
@@ -6901,6 +6954,8 @@
     <mergeCell ref="A62:O62"/>
     <mergeCell ref="A63:O63"/>
     <mergeCell ref="A64:O64"/>
+    <mergeCell ref="A65:O65"/>
+    <mergeCell ref="A76:G76"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>